<commit_message>
Update CO2 laser questionnaire link and estimate breakdown
</commit_message>
<xml_diff>
--- a/outputs/mirai-clinic-updates/みらい内科クリニック 美容サイト改修 見積切り分け表.xlsx
+++ b/outputs/mirai-clinic-updates/みらい内科クリニック 美容サイト改修 見積切り分け表.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="1" r:id="Rb6922cdd15b34f12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積対象内" sheetId="2" r:id="R111461e762d14673"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積対象外" sheetId="3" r:id="Rc838a1d693de459f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メール一覧" sheetId="4" r:id="R5891f87f36324303"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="1" r:id="R5aa997a062964587"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積対象内" sheetId="2" r:id="Ra3c5e27ba5f34c76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積対象外" sheetId="3" r:id="Rb8a66714405b4a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メール一覧" sheetId="4" r:id="R74e7f7c406e54b62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37,9 +37,6 @@
     <x:t xml:space="preserve">見積対象外 件数</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">20件＋直近1週間追加分7件（既存表の下に追加）</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">切り分け基準</x:t>
   </x:si>
   <x:si>
@@ -74,9 +71,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">小計値の注意</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Notionの小計行は再分類後に再計算されていないため、本表では各シートに「（参考）再計算合計」を併記しています。追加依頼（美容修正P1〜P3、ダイエット修正）を反映済み。</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">備考</x:t>
@@ -547,6 +541,31 @@
     <x:t xml:space="preserve">美容修正P3</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">美容問診票PDF差し替え、マッサージピール・リバースピール同意書追加、全ページの書類カード配色統一・下線削除</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">添付PDF差し替え、同意書配置、全ページの問診票・同意書カードの配色統一を反映。</x:t>
+  </x:si>
+  <x:si>
+    <x:r>
+      <x:rPr>
+        <x:sz val="1000"/>
+        <x:color rgb="FF1155CC"/>
+        <x:rFont val="MS Gothic"/>
+        <x:family val="2"/>
+      </x:rPr>
+      <x:t xml:space="preserve">美容修正</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:sz val="1000"/>
+        <x:color rgb="FF1155CC"/>
+        <x:rFont val="Arial"/>
+      </x:rPr>
+      <x:t xml:space="preserve">P3</x:t>
+    </x:r>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">ダイエット修正</x:t>
   </x:si>
   <x:si>
@@ -649,10 +668,112 @@
     <x:t xml:space="preserve">6月28日のダイエットの件</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">見積対象外</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">既存ページ修正、文言差し替え、価格表差し替え、MENU/FAQ削除、注意事項追加、画像・添付差し替え等</x:t>
+    <x:t xml:space="preserve">2026-07-10</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">ウルティムガン追加修正</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">施術詳細・料金表・ラインナップ・同意書カードの修正</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">既存ページの文言・構成・書類導線・カード配色を修正。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">添付画像（2026-07-10）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美容サイト ②（リフテラV）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">表題変更、施術詳細・副作用・注意点・施術不可条件の更新、新同意書への差し替え</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">メール件名: 美容サイト ②。TDTテクノロジー後の詳細セクション追加を含む。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">2026-07-10 受信</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美容サイト ③（ピアモリフティング）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">表題・MENU表記・詳細・施術不可条件の更新、料金表削除、新同意書差し替え、価格表表記修正</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">メール件名: 美容サイト ③。美肌治療価格表内のボディ表記修正を含む。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美容サイト ④（ダーマペン4）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">施術詳細の並び・文言更新、ラインナップ見出し変更・並び替え、施術不可条件更新、注意項目削除、新同意書差し替え</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">メール件名: 美容サイト ④。施術時に注意が必要な方セクションの削除を含む。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美肌サイト ⑤（炭酸ガスレーザー）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">表題・施術不可見出しの変更、料金削除、アフターケア文言更新、美肌治療価格表の表示内容更新</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">メール件名: 美容サイト ⑤。ほくろ・首イボの価格表を含む。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美肌サイト ⑥（タトゥー除去）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">日焼け注意文の修正、説明文修正、注意事項・副作用・リスクの再構成、施術不可条件の追加</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">メール件名: 美肌サイト ⑥。タトゥー除去レーザーのリスクセクション削除を含む。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美肌サイト ⑦（レーザーフェイシャル）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">表題デザイン・説明文の更新、施術詳細・注意事項・副作用・リスクなどの追加</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">メール件名: 美肌サイト ⑦。対象症状、施術時間、注意事項の追加を含む。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美肌サイト ⑧（YAGレーザーシャワー）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">メール件名: 美肌サイト ⑧。対象症状、施術時間、注意事項の追加を含む。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美肌サイト ⑨（YAGリフトアップレーザー）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">メール件名: 美肌サイト ⑨。対象症状、施術時間、注意事項の追加を含む。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">2026-07-16</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">修正後の修正①</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">マッサージピールの項目順を変更。サーマニードルEVO・ピアモリフティングの美肌治療価格表をスマホ縦画面で見やすく調整</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">既存ページの項目並び替え・既存価格表のモバイル表示調整。新規サービス追加は含まれない。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">2026-07-16 受信</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">修正後の修正②</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">CO2レーザーのスマホ表示、共通価格表の回数表記、全施術の書類カード書体・表記・保護者同意書・問診票、FAQ表示を修正</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">既存ページの表示・書体・文言・価格表・書類カード・FAQの統一。新規サービス追加は含まれない。</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">日付</x:t>
@@ -788,13 +909,19 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">マンジャロ削除、ゼップバウンドへ変更</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">マッサージピールの項目順、サーマニードルEVO・ピアモのスマホ表示調整</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">CO2・共通価格表・書類カード・保護者同意書・FAQの修正</x:t>
   </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="15">
+  <x:fonts count="18">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -855,6 +982,10 @@
       <x:name val="Arial"/>
     </x:font>
     <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
       <x:sz val="409"/>
       <x:color rgb="FF1155CC"/>
       <x:name val="MS Gothic"/>
@@ -867,6 +998,16 @@
     <x:font>
       <x:sz val="6"/>
       <x:name val="07NikumaruFont"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1155CC"/>
+      <x:name val="MS Gothic"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1155CC"/>
+      <x:name val="Arial"/>
     </x:font>
   </x:fonts>
   <x:fills count="6">
@@ -918,7 +1059,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="21">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -960,6 +1101,18 @@
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1190,7 +1343,7 @@
     <x:col min="2" max="2" width="80" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="24" customHeight="1">
+    <x:row r="1" ht="42.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -1227,8 +1380,8 @@
       <x:c r="A6" s="2" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>8</x:v>
+      <x:c r="B6" s="3" t="str">
+        <x:v>41件（修正後の修正③〜⑦を含む）</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1237,64 +1390,64 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B8" s="3"/>
+    </x:row>
+    <x:row r="9" ht="66.25" customHeight="1">
+      <x:c r="A9" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B8" s="3"/>
-    </x:row>
-    <x:row r="9" ht="37.25" customHeight="1">
-      <x:c r="A9" s="2" t="s">
+      <x:c r="B9" s="3" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B9" s="3" t="s">
+    </x:row>
+    <x:row r="10" ht="66.25" customHeight="1">
+      <x:c r="A10" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="37.25" customHeight="1">
-      <x:c r="A10" s="2" t="s">
+      <x:c r="B10" s="3" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B10" s="3" t="s">
+    </x:row>
+    <x:row r="11" ht="66.25" customHeight="1">
+      <x:c r="A11" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="37.25" customHeight="1">
-      <x:c r="A11" s="2" t="s">
+      <x:c r="B11" s="3" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B11" s="3" t="s">
+    </x:row>
+    <x:row r="12" ht="66.25" customHeight="1">
+      <x:c r="A12" s="2" t="s">
         <x:v>15</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="37.25" customHeight="1">
-      <x:c r="A12" s="2" t="s">
+      <x:c r="B12" s="3" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B12" s="3" t="s">
+    </x:row>
+    <x:row r="13" ht="66.25" customHeight="1">
+      <x:c r="A13" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="37.25" customHeight="1">
-      <x:c r="A13" s="2" t="s">
+      <x:c r="B13" s="3" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B13" s="3" t="s">
+    </x:row>
+    <x:row r="14" ht="66.25" customHeight="1">
+      <x:c r="A14" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="37.25" customHeight="1">
-      <x:c r="A14" s="2" t="s">
+      <x:c r="B14" s="20" t="str">
+        <x:v>Notionの小計行は既存の修正依頼を反映済み。今回、最新メールの「修正後の修正③〜⑦」を追記（⑦は一部対応済み・残件要確認）。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="66.25" customHeight="1">
+      <x:c r="A15" s="2" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B14" s="3" t="s">
+      <x:c r="B15" s="3" t="s">
         <x:v>21</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="37.25" customHeight="1">
-      <x:c r="A15" s="2" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B15" s="3" t="s">
-        <x:v>23</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1316,541 +1469,541 @@
     <x:col min="8" max="8" width="26" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="20" customHeight="1">
+    <x:row r="1" ht="35.75" customHeight="1">
       <x:c r="A1" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="s">
+      <x:c r="D1" s="4" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="s">
+      <x:c r="E1" s="4" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="s">
+      <x:c r="F1" s="13" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="s">
+      <x:c r="G1" s="4" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="F1" s="13" t="s">
+      <x:c r="H1" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="s">
+    </x:row>
+    <x:row r="2" ht="66.25" customHeight="1">
+      <x:c r="A2" s="5" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="s">
+      <x:c r="B2" s="5" t="s">
         <x:v>31</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="37.25" customHeight="1">
-      <x:c r="A2" s="5" t="s">
+      <x:c r="C2" s="5" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C2" s="5" t="s">
+      <x:c r="D2" s="5" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E2" s="5" t="s">
         <x:v>34</x:v>
-      </x:c>
-      <x:c r="D2" s="5" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E2" s="5" t="s">
-        <x:v>36</x:v>
       </x:c>
       <x:c r="F2" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G2" s="5" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="H2" s="6" t="s">
+        <x:v>31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="66.25" customHeight="1">
+      <x:c r="A3" s="5" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B3" s="5" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="C3" s="5" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="H2" s="6" t="s">
-        <x:v>33</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="37.25" customHeight="1">
-      <x:c r="A3" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B3" s="5" t="s">
+      <x:c r="D3" s="5" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D3" s="5" t="s">
-        <x:v>40</x:v>
-      </x:c>
       <x:c r="E3" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F3" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G3" s="5" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="H3" s="6" t="s">
+        <x:v>36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="66.25" customHeight="1">
+      <x:c r="A4" s="5" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="H3" s="6" t="s">
-        <x:v>38</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="37.25" customHeight="1">
-      <x:c r="A4" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="s">
+      <x:c r="D4" s="5" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="s">
-        <x:v>44</x:v>
-      </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F4" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G4" s="5" t="s">
-        <x:v>45</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="H4" s="6" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="5" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>46</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F5" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="5" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="s">
+        <x:v>44</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="66.25" customHeight="1">
+      <x:c r="A6" s="5" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="H5" s="6" t="s">
-        <x:v>46</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="37.25" customHeight="1">
-      <x:c r="A6" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B6" s="5" t="s">
+      <x:c r="D6" s="5" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>51</x:v>
-      </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F6" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="5" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="s">
+        <x:v>51</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="66.25" customHeight="1">
+      <x:c r="A7" s="5" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="H6" s="6" t="s">
+      <x:c r="B7" s="5" t="s">
         <x:v>53</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="37.25" customHeight="1">
-      <x:c r="A7" s="5" t="s">
+      <x:c r="C7" s="5" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="s">
+      <x:c r="D7" s="5" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="s">
-        <x:v>57</x:v>
-      </x:c>
       <x:c r="E7" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F7" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G7" s="5" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="s">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="66.25" customHeight="1">
+      <x:c r="A8" s="5" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="H7" s="6" t="s">
-        <x:v>55</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="37.25" customHeight="1">
-      <x:c r="A8" s="5" t="s">
+      <x:c r="C8" s="5" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="s">
+      <x:c r="D8" s="5" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>62</x:v>
-      </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F8" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G8" s="5" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="s">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="66.25" customHeight="1">
+      <x:c r="A9" s="5" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="H8" s="6" t="s">
+      <x:c r="B9" s="5" t="s">
         <x:v>64</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="37.25" customHeight="1">
-      <x:c r="A9" s="5" t="s">
+      <x:c r="C9" s="5" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="s">
+      <x:c r="D9" s="5" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="C9" s="5" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="s">
-        <x:v>68</x:v>
-      </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F9" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="H9" s="6" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="5" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>73</x:v>
-      </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F10" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="5" t="s">
-        <x:v>74</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="H10" s="6" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B11" s="5" t="s">
-        <x:v>75</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C11" s="5" t="s">
-        <x:v>76</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D11" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F11" s="10">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G11" s="5" t="s">
-        <x:v>77</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="H11" s="6" t="s">
-        <x:v>75</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>78</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>79</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D12" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F12" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G12" s="5" t="s">
-        <x:v>80</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H12" s="6" t="s">
-        <x:v>78</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
-        <x:v>81</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C13" s="5" t="s">
-        <x:v>82</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D13" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F13" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="5" t="s">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="H13" s="6" t="s">
-        <x:v>81</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="5" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B14" s="5" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="C14" s="5" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="B14" s="5" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>86</x:v>
-      </x:c>
       <x:c r="D14" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F14" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G14" s="5" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="s">
+        <x:v>83</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="66.25" customHeight="1">
+      <x:c r="A15" s="5" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="B15" s="5" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="H14" s="6" t="s">
-        <x:v>85</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="37.25" customHeight="1">
-      <x:c r="A15" s="5" t="s">
+      <x:c r="C15" s="5" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="B15" s="5" t="s">
-        <x:v>89</x:v>
-      </x:c>
-      <x:c r="C15" s="5" t="s">
-        <x:v>90</x:v>
-      </x:c>
       <x:c r="D15" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E15" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F15" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G15" s="5" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="H15" s="6" t="s">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="66.25" customHeight="1">
+      <x:c r="A16" s="5" t="s">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="H15" s="6" t="s">
+      <x:c r="B16" s="5" t="s">
         <x:v>92</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="37.25" customHeight="1">
-      <x:c r="A16" s="5" t="s">
+      <x:c r="C16" s="5" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="C16" s="5" t="s">
-        <x:v>95</x:v>
-      </x:c>
       <x:c r="D16" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F16" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G16" s="5" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="s">
+        <x:v>92</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="66.25" customHeight="1">
+      <x:c r="A17" s="5" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="B17" s="5" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="C17" s="5" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="H16" s="6" t="s">
-        <x:v>94</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="37.25" customHeight="1">
-      <x:c r="A17" s="5" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="B17" s="5" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="C17" s="5" t="s">
-        <x:v>98</x:v>
-      </x:c>
       <x:c r="D17" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E17" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F17" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G17" s="5" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="H17" s="6" t="s">
+        <x:v>95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="66.25" customHeight="1">
+      <x:c r="A18" s="5" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="s">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="H17" s="6" t="s">
-        <x:v>97</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="37.25" customHeight="1">
-      <x:c r="A18" s="5" t="s">
+      <x:c r="C18" s="5" t="s">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="B18" s="5" t="s">
-        <x:v>101</x:v>
-      </x:c>
-      <x:c r="C18" s="5" t="s">
-        <x:v>102</x:v>
-      </x:c>
       <x:c r="D18" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E18" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F18" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G18" s="5" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="H18" s="6" t="s">
+        <x:v>99</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="99.75" customHeight="1">
+      <x:c r="A19" s="5" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B19" s="5" t="s">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="H18" s="6" t="s">
-        <x:v>101</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="56" customHeight="1">
-      <x:c r="A19" s="5" t="s">
+      <x:c r="C19" s="5" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="B19" s="5" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="C19" s="5" t="s">
-        <x:v>106</x:v>
-      </x:c>
       <x:c r="D19" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E19" s="12" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F19" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="5" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="H19" s="6" t="s">
+        <x:v>103</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="99.75" customHeight="1">
+      <x:c r="A20" s="5" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="B20" s="5" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="H19" s="6" t="s">
-        <x:v>105</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="56" customHeight="1">
-      <x:c r="A20" s="5" t="s">
+      <x:c r="C20" s="5" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="B20" s="5" t="s">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="C20" s="5" t="s">
-        <x:v>110</x:v>
-      </x:c>
       <x:c r="D20" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E20" s="12" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F20" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G20" s="5" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="H20" s="6" t="s">
+        <x:v>107</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="66.25" customHeight="1">
+      <x:c r="A21" s="7" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="s">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="H20" s="6" t="s">
-        <x:v>109</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="37.25" customHeight="1">
-      <x:c r="A21" s="7" t="s">
+      <x:c r="C21" s="7" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="B21" s="7" t="s">
+      <x:c r="D21" s="7" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="C21" s="7" t="s">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="D21" s="7" t="s">
-        <x:v>115</x:v>
-      </x:c>
       <x:c r="E21" s="7" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F21" s="7" t="n">
         <x:f>SUM(F2:F20)</x:f>
@@ -1861,25 +2014,25 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="R8219993ff89646ec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="R4fdfeb4863af4dc3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="R6706d52813cb4608"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="R15625582d0ee49ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="Rad00e31e611d488f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="R8b783eba672d4c53"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="R65774368a2a54ff5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R7a59a75c6df14519"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="Rbcbfeffeaaf34501"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="R90f5edfff795482f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R70153870055b4cf4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="R94d7bc98b5c6418d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Rc77db5ec17a64c43"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="Raf2b9a29f9874fd0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="Rc1ab143861c74bb2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="R41d3b8a6dfe64ad1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="R5967dfd185fc424d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="R0145b00551bb49b7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R01d26c18ebf7479e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="R4d4bb2da9b1c4228"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="Ra9e1dddd3ecc48f6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="R6231fd0a4d9045b3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="Rca791d064a44464c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R0a5ab329a9694c1f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rc18e353e40d84316"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="R7534dcb02ef94ab8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R05c65a96865b462b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="Rc02b69d857344427"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="Rf30e7d35b136425a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R6a2d3ec3be1a44f1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="R98dc4b6b632d4e17"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Red81e1b966344068"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="Rcaaded9020be4d78"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="Ref1bd6d1220543ed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="Ra44f0391cca040c9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="Re92130abeb1d4934"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="R573a4caa513149b2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R772b86e931a34c35"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1899,946 +2052,1168 @@
     <x:col min="8" max="8" width="26" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="20" customHeight="1">
+    <x:row r="1" ht="35.75" customHeight="1">
       <x:c r="A1" s="8" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C1" s="8" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B1" s="8" t="s">
+      <x:c r="D1" s="8" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="C1" s="8" t="s">
+      <x:c r="E1" s="8" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D1" s="8" t="s">
+      <x:c r="F1" s="11" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E1" s="8" t="s">
+      <x:c r="G1" s="8" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="F1" s="11" t="s">
+      <x:c r="H1" s="8" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="G1" s="8" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="H1" s="8" t="s">
-        <x:v>31</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="56" customHeight="1">
+    </x:row>
+    <x:row r="2" ht="99.75" customHeight="1">
       <x:c r="A2" s="5" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="B2" s="5" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="C2" s="5" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="s">
+      <x:c r="D2" s="5" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="s">
         <x:v>117</x:v>
-      </x:c>
-      <x:c r="C2" s="5" t="s">
-        <x:v>118</x:v>
-      </x:c>
-      <x:c r="D2" s="5" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E2" s="12" t="s">
-        <x:v>119</x:v>
       </x:c>
       <x:c r="F2" s="10">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G2" s="5" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="H2" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="66.25" customHeight="1">
+      <x:c r="A3" s="5" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="B3" s="5" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="H2" s="6" t="s">
+      <x:c r="C3" s="5" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="D3" s="5" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E3" s="5" t="s">
         <x:v>117</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="37.25" customHeight="1">
-      <x:c r="A3" s="5" t="s">
-        <x:v>121</x:v>
-      </x:c>
-      <x:c r="B3" s="5" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="C3" s="5" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="D3" s="5" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E3" s="5" t="s">
-        <x:v>119</x:v>
       </x:c>
       <x:c r="F3" s="10">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G3" s="5" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="H3" s="6" t="s">
+        <x:v>123</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="133" customHeight="1">
+      <x:c r="A4" s="5" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="H3" s="6" t="s">
+      <x:c r="C4" s="5" t="s">
         <x:v>125</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="74.75" customHeight="1">
-      <x:c r="A4" s="5" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="s">
-        <x:v>127</x:v>
-      </x:c>
       <x:c r="D4" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F4" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G4" s="5" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="s">
+        <x:v>124</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="66.25" customHeight="1">
+      <x:c r="A5" s="5" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B5" s="5" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="C5" s="5" t="s">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="H4" s="6" t="s">
-        <x:v>126</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="37.25" customHeight="1">
-      <x:c r="A5" s="5" t="s">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="B5" s="5" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="C5" s="5" t="s">
-        <x:v>130</x:v>
-      </x:c>
       <x:c r="D5" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F5" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G5" s="5" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="s">
+        <x:v>127</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="66.25" customHeight="1">
+      <x:c r="A6" s="5" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
         <x:v>131</x:v>
       </x:c>
-      <x:c r="H5" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="37.25" customHeight="1">
-      <x:c r="A6" s="5" t="s">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="B6" s="5" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="s">
-        <x:v>133</x:v>
-      </x:c>
       <x:c r="D6" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F6" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G6" s="5" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="s">
+        <x:v>130</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="35.75" customHeight="1">
+      <x:c r="A7" s="5" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="C7" s="5" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="H6" s="6" t="s">
-        <x:v>132</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="20" customHeight="1">
-      <x:c r="A7" s="5" t="s">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="B7" s="5" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="C7" s="5" t="s">
-        <x:v>136</x:v>
-      </x:c>
       <x:c r="D7" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E7" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F7" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G7" s="5" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="s">
+        <x:v>133</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="66.25" customHeight="1">
+      <x:c r="A8" s="5" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="H7" s="6" t="s">
-        <x:v>135</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="37.25" customHeight="1">
-      <x:c r="A8" s="5" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="B8" s="5" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>139</x:v>
-      </x:c>
       <x:c r="D8" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F8" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G8" s="5" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="s">
+        <x:v>136</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="66.25" customHeight="1">
+      <x:c r="A9" s="5" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="C9" s="5" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="H8" s="6" t="s">
-        <x:v>138</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="37.25" customHeight="1">
-      <x:c r="A9" s="5" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="B9" s="5" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="C9" s="5" t="s">
-        <x:v>142</x:v>
-      </x:c>
       <x:c r="D9" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F9" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G9" s="5" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="s">
+        <x:v>139</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="35.75" customHeight="1">
+      <x:c r="A10" s="5" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="H9" s="6" t="s">
-        <x:v>141</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="20" customHeight="1">
-      <x:c r="A10" s="5" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="B10" s="5" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>145</x:v>
-      </x:c>
       <x:c r="D10" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F10" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G10" s="5" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="s">
+        <x:v>142</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="66.25" customHeight="1">
+      <x:c r="A11" s="5" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="C11" s="5" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="H10" s="6" t="s">
-        <x:v>144</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="37.25" customHeight="1">
-      <x:c r="A11" s="5" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="B11" s="5" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C11" s="5" t="s">
-        <x:v>148</x:v>
-      </x:c>
       <x:c r="D11" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F11" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G11" s="5" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="s">
+        <x:v>145</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="66.25" customHeight="1">
+      <x:c r="A12" s="5" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="H11" s="6" t="s">
-        <x:v>147</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="37.25" customHeight="1">
-      <x:c r="A12" s="5" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="B12" s="5" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>151</x:v>
-      </x:c>
       <x:c r="D12" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F12" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G12" s="5" t="s">
-        <x:v>149</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="H12" s="6" t="s">
+        <x:v>148</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="66.25" customHeight="1">
+      <x:c r="A13" s="5" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B13" s="5" t="s">
         <x:v>150</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="37.25" customHeight="1">
-      <x:c r="A13" s="5" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="B13" s="5" t="s">
-        <x:v>152</x:v>
-      </x:c>
       <x:c r="C13" s="5" t="s">
-        <x:v>153</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="D13" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F13" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G13" s="5" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="s">
+        <x:v>150</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="99.75" customHeight="1">
+      <x:c r="A14" s="5" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B14" s="5" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="C14" s="5" t="s">
         <x:v>154</x:v>
       </x:c>
-      <x:c r="H13" s="6" t="s">
-        <x:v>152</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="56" customHeight="1">
-      <x:c r="A14" s="5" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="B14" s="5" t="s">
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>156</x:v>
-      </x:c>
       <x:c r="D14" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F14" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G14" s="5" t="s">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="s">
+        <x:v>153</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="66.25" customHeight="1">
+      <x:c r="A15" s="5" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="B15" s="5" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="C15" s="5" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="H14" s="6" t="s">
-        <x:v>155</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="37.25" customHeight="1">
-      <x:c r="A15" s="5" t="s">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="B15" s="5" t="s">
-        <x:v>158</x:v>
-      </x:c>
-      <x:c r="C15" s="5" t="s">
-        <x:v>159</x:v>
-      </x:c>
       <x:c r="D15" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E15" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F15" s="5">
         <x:v>3</x:v>
       </x:c>
       <x:c r="G15" s="5" t="s">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="H15" s="6" t="s">
+        <x:v>156</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="99.75" customHeight="1">
+      <x:c r="A16" s="5" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="B16" s="5" t="s">
         <x:v>160</x:v>
       </x:c>
-      <x:c r="H15" s="6" t="s">
-        <x:v>158</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="56" customHeight="1">
-      <x:c r="A16" s="5" t="s">
+      <x:c r="C16" s="5" t="s">
         <x:v>161</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="s">
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="C16" s="5" t="s">
-        <x:v>163</x:v>
-      </x:c>
       <x:c r="D16" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F16" s="5">
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="G16" s="5" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="s">
+        <x:v>160</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="66.25" customHeight="1">
+      <x:c r="A17" s="5" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="B17" s="5" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="C17" s="5" t="s">
         <x:v>164</x:v>
       </x:c>
-      <x:c r="H16" s="6" t="s">
-        <x:v>162</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="37.25" customHeight="1">
-      <x:c r="A17" s="5" t="s">
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="B17" s="5" t="s">
+      <x:c r="D17" s="5" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="C17" s="5" t="s">
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="D17" s="5" t="s">
-        <x:v>167</x:v>
-      </x:c>
       <x:c r="E17" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F17" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G17" s="5" t="s">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="H17" s="16" t="s">
+        <x:v>167</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="66.25" customHeight="1">
+      <x:c r="A18" s="5" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="H17" s="16" t="s">
+      <x:c r="B18" s="5" t="s">
         <x:v>169</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="37.25" customHeight="1">
-      <x:c r="A18" s="5" t="s">
+      <x:c r="C18" s="5" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="B18" s="5" t="s">
+      <x:c r="D18" s="5" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E18" s="5" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F18" s="5">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G18" s="5" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="C18" s="5" t="str">
-        <x:v>美容問診票PDF差し替え、マッサージピール・リバースピール同意書追加、全ページの書類カード配色統一・下線削除</x:v>
-      </x:c>
-      <x:c r="D18" s="5" t="str">
-        <x:v>対応済み</x:v>
-      </x:c>
-      <x:c r="E18" s="5" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F18" s="5" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G18" s="5" t="str">
-        <x:v>添付PDF差し替え、同意書配置、全ページの問診票・同意書カードの配色統一を反映。</x:v>
-      </x:c>
-      <x:c r="H18" s="6" t="s">
-        <x:v>171</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="37.25" customHeight="1">
+      <x:c r="H18" s="18" t="s">
+        <x:v>172</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="66.25" customHeight="1">
       <x:c r="A19" s="5" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="C19" s="5" t="s">
-        <x:v>173</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="D19" s="12" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E19" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F19" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="5" t="s">
-        <x:v>174</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="H19" s="6" t="s">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28">
       <x:c r="A20" s="5" t="s">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
-        <x:v>177</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C20" s="5" t="s">
-        <x:v>178</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="D20" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E20" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F20" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G20" s="5" t="s">
-        <x:v>179</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="H20" s="15" t="s">
-        <x:v>180</x:v>
+        <x:v>181</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="28">
       <x:c r="A21" s="5" t="s">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B21" s="5" t="s">
-        <x:v>181</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C21" s="5" t="s">
-        <x:v>182</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="D21" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E21" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F21" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G21" s="5" t="s">
-        <x:v>183</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="H21" s="15" t="s">
-        <x:v>184</x:v>
+        <x:v>185</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28">
       <x:c r="A22" s="5" t="s">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
-        <x:v>185</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="C22" s="5" t="s">
-        <x:v>186</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="D22" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E22" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F22" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G22" s="5" t="s">
-        <x:v>187</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="H22" s="15" t="s">
-        <x:v>188</x:v>
+        <x:v>189</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42">
       <x:c r="A23" s="5" t="s">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
-        <x:v>189</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="C23" s="5" t="s">
-        <x:v>190</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="D23" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E23" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F23" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G23" s="5" t="s">
-        <x:v>191</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="H23" s="15" t="s">
-        <x:v>192</x:v>
+        <x:v>193</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42">
       <x:c r="A24" s="5" t="s">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
-        <x:v>193</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C24" s="5" t="s">
-        <x:v>194</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D24" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E24" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F24" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G24" s="5" t="s">
-        <x:v>195</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="H24" s="15" t="s">
-        <x:v>196</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42">
       <x:c r="A25" s="5" t="s">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
-        <x:v>197</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C25" s="5" t="s">
-        <x:v>198</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="D25" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E25" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F25" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G25" s="5" t="s">
-        <x:v>199</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="H25" s="15" t="s">
-        <x:v>200</x:v>
+        <x:v>201</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28">
       <x:c r="A26" s="5" t="s">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="B26" s="5" t="s">
-        <x:v>202</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C26" s="5" t="s">
-        <x:v>203</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D26" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E26" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F26" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G26" s="5" t="s">
-        <x:v>204</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="H26" s="15" t="s">
-        <x:v>205</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" t="str">
-        <x:v>2026-07-10</x:v>
-      </x:c>
-      <x:c r="B27" t="str">
-        <x:v>ウルティムガン追加修正</x:v>
-      </x:c>
-      <x:c r="C27" t="str">
-        <x:v>施術詳細・料金表・ラインナップ・同意書カードの修正</x:v>
-      </x:c>
-      <x:c r="D27" t="str">
-        <x:v>対応済み</x:v>
-      </x:c>
-      <x:c r="E27" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F27" t="n">
+        <x:v>206</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="53.25" customHeight="1">
+      <x:c r="A27" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B27" t="s">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="C27" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="D27" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E27" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F27">
         <x:v>2.5</x:v>
       </x:c>
-      <x:c r="G27" t="str">
-        <x:v>既存ページの文言・構成・書類導線・カード配色を修正。</x:v>
-      </x:c>
-      <x:c r="H27" t="str">
-        <x:v>添付画像（2026-07-10）</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="42" customHeight="1">
-      <x:c r="A28" t="str">
-        <x:v>2026-07-10</x:v>
-      </x:c>
-      <x:c r="B28" t="str">
-        <x:v>美容サイト ②（リフテラV）</x:v>
-      </x:c>
-      <x:c r="C28" t="str">
-        <x:v>表題変更、施術詳細・副作用・注意点・施術不可条件の更新、新同意書への差し替え</x:v>
-      </x:c>
-      <x:c r="D28" t="str">
-        <x:v>未対応</x:v>
-      </x:c>
-      <x:c r="E28" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F28" t="str"/>
-      <x:c r="G28" t="str">
-        <x:v>メール件名: 美容サイト ②。TDTテクノロジー後の詳細セクション追加を含む。</x:v>
-      </x:c>
-      <x:c r="H28" t="str">
-        <x:v>2026-07-10 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="42" customHeight="1">
-      <x:c r="A29" t="str">
-        <x:v>2026-07-10</x:v>
-      </x:c>
-      <x:c r="B29" t="str">
-        <x:v>美容サイト ③（ピアモリフティング）</x:v>
-      </x:c>
-      <x:c r="C29" t="str">
-        <x:v>表題・MENU表記・詳細・施術不可条件の更新、料金表削除、新同意書差し替え、価格表表記修正</x:v>
-      </x:c>
-      <x:c r="D29" t="str">
-        <x:v>未対応</x:v>
-      </x:c>
-      <x:c r="E29" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F29" t="str"/>
-      <x:c r="G29" t="str">
-        <x:v>メール件名: 美容サイト ③。美肌治療価格表内のボディ表記修正を含む。</x:v>
-      </x:c>
-      <x:c r="H29" t="str">
-        <x:v>2026-07-10 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="42" customHeight="1">
-      <x:c r="A30" t="str">
-        <x:v>2026-07-10</x:v>
-      </x:c>
-      <x:c r="B30" t="str">
-        <x:v>美容サイト ④（ダーマペン4）</x:v>
-      </x:c>
-      <x:c r="C30" t="str">
-        <x:v>施術詳細の並び・文言更新、ラインナップ見出し変更・並び替え、施術不可条件更新、注意項目削除、新同意書差し替え</x:v>
-      </x:c>
-      <x:c r="D30" t="str">
-        <x:v>未対応</x:v>
-      </x:c>
-      <x:c r="E30" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F30" t="str"/>
-      <x:c r="G30" t="str">
-        <x:v>メール件名: 美容サイト ④。施術時に注意が必要な方セクションの削除を含む。</x:v>
-      </x:c>
-      <x:c r="H30" t="str">
-        <x:v>2026-07-10 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="42" customHeight="1">
-      <x:c r="A31" t="str">
-        <x:v>2026-07-10</x:v>
-      </x:c>
-      <x:c r="B31" t="str">
-        <x:v>美肌サイト ⑤（炭酸ガスレーザー）</x:v>
-      </x:c>
-      <x:c r="C31" t="str">
-        <x:v>表題・施術不可見出しの変更、料金削除、アフターケア文言更新、美肌治療価格表の表示内容更新</x:v>
-      </x:c>
-      <x:c r="D31" t="str">
-        <x:v>未対応</x:v>
-      </x:c>
-      <x:c r="E31" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F31" t="str"/>
-      <x:c r="G31" t="str">
-        <x:v>メール件名: 美容サイト ⑤。ほくろ・首イボの価格表を含む。</x:v>
-      </x:c>
-      <x:c r="H31" t="str">
-        <x:v>2026-07-10 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="42" customHeight="1">
-      <x:c r="A32" t="str">
-        <x:v>2026-07-10</x:v>
-      </x:c>
-      <x:c r="B32" t="str">
-        <x:v>美肌サイト ⑥（タトゥー除去）</x:v>
-      </x:c>
-      <x:c r="C32" t="str">
-        <x:v>日焼け注意文の修正、説明文修正、注意事項・副作用・リスクの再構成、施術不可条件の追加</x:v>
-      </x:c>
-      <x:c r="D32" t="str">
-        <x:v>未対応</x:v>
-      </x:c>
-      <x:c r="E32" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F32" t="str"/>
-      <x:c r="G32" t="str">
-        <x:v>メール件名: 美肌サイト ⑥。タトゥー除去レーザーのリスクセクション削除を含む。</x:v>
-      </x:c>
-      <x:c r="H32" t="str">
-        <x:v>2026-07-10 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="42" customHeight="1">
-      <x:c r="A33" t="str">
-        <x:v>2026-07-10</x:v>
-      </x:c>
-      <x:c r="B33" t="str">
-        <x:v>美肌サイト ⑦（レーザーフェイシャル）</x:v>
-      </x:c>
-      <x:c r="C33" t="str">
-        <x:v>表題デザイン・説明文の更新、施術詳細・注意事項・副作用・リスクなどの追加</x:v>
-      </x:c>
-      <x:c r="D33" t="str">
-        <x:v>未対応</x:v>
-      </x:c>
-      <x:c r="E33" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F33" t="str"/>
-      <x:c r="G33" t="str">
-        <x:v>メール件名: 美肌サイト ⑦。対象症状、施術時間、注意事項の追加を含む。</x:v>
-      </x:c>
-      <x:c r="H33" t="str">
-        <x:v>2026-07-10 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="42" customHeight="1">
-      <x:c r="A34" t="str">
-        <x:v>2026-07-10</x:v>
-      </x:c>
-      <x:c r="B34" t="str">
-        <x:v>美肌サイト ⑧（YAGレーザーシャワー）</x:v>
-      </x:c>
-      <x:c r="C34" t="str">
-        <x:v>表題デザイン・説明文の更新、施術詳細・注意事項・副作用・リスクなどの追加</x:v>
-      </x:c>
-      <x:c r="D34" t="str">
-        <x:v>未対応</x:v>
-      </x:c>
-      <x:c r="E34" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F34" t="str"/>
-      <x:c r="G34" t="str">
-        <x:v>メール件名: 美肌サイト ⑧。対象症状、施術時間、注意事項の追加を含む。</x:v>
-      </x:c>
-      <x:c r="H34" t="str">
-        <x:v>2026-07-10 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="42" customHeight="1">
-      <x:c r="A35" t="str">
-        <x:v>2026-07-10</x:v>
-      </x:c>
-      <x:c r="B35" t="str">
-        <x:v>美肌サイト ⑨（YAGリフトアップレーザー）</x:v>
-      </x:c>
-      <x:c r="C35" t="str">
-        <x:v>表題デザイン・説明文の更新、施術詳細・注意事項・副作用・リスクなどの追加</x:v>
-      </x:c>
-      <x:c r="D35" t="str">
-        <x:v>未対応</x:v>
-      </x:c>
-      <x:c r="E35" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F35" t="str"/>
-      <x:c r="G35" t="str">
-        <x:v>メール件名: 美肌サイト ⑨。対象症状、施術時間、注意事項の追加を含む。</x:v>
-      </x:c>
-      <x:c r="H35" t="str">
-        <x:v>2026-07-10 受信</x:v>
+      <x:c r="G27" t="s">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="H27" t="s">
+        <x:v>211</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="29.25" customHeight="1">
+      <x:c r="A28" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B28" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="C28" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="D28" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E28" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F28" s="17">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G28" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="H28" t="s">
+        <x:v>215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="36" customHeight="1">
+      <x:c r="A29" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B29" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="C29" t="s">
+        <x:v>217</x:v>
+      </x:c>
+      <x:c r="D29" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E29" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F29" s="17">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G29" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="H29" t="s">
+        <x:v>215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="40" customHeight="1">
+      <x:c r="A30" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B30" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="C30" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="D30" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E30" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F30" s="17">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G30" t="s">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="H30" t="s">
+        <x:v>215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="36" customHeight="1">
+      <x:c r="A31" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B31" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="C31" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="D31" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E31" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F31" s="17">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G31" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H31" t="s">
+        <x:v>215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="33.25" customHeight="1">
+      <x:c r="A32" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B32" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="C32" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="D32" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E32" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F32" s="17">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G32" t="s">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="H32" t="s">
+        <x:v>215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="36" customHeight="1">
+      <x:c r="A33" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B33" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="C33" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="D33" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E33" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F33" s="17">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G33" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="H33" t="s">
+        <x:v>215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="20" customHeight="1">
+      <x:c r="A34" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B34" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="C34" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="D34" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E34" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F34" s="17">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G34" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="H34" t="s">
+        <x:v>215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B35" t="s">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c r="C35" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="D35" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E35" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F35" s="17">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G35" t="s">
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="H35" t="s">
+        <x:v>215</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="s">
-        <x:v>112</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="B36" t="s">
-        <x:v>206</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C36" t="s">
-        <x:v>207</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="D36" t="s">
-        <x:v>115</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E36" t="s">
-        <x:v>119</x:v>
-      </x:c>
-      <x:c r="F36" t="n">
-        <x:f>SUM(F2:F35)</x:f>
-        <x:v>32.5</x:v>
-      </x:c>
-      <x:c r="G36"/>
-      <x:c r="H36"/>
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F36">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="G36" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="H36" t="s">
+        <x:v>239</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="B37" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C37" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D37" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E37" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F37">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="G37" t="s">
+        <x:v>242</x:v>
+      </x:c>
+      <x:c r="H37" t="s">
+        <x:v>239</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="56" customHeight="1">
+      <x:c r="A38" s="19" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="B38" s="19" t="str">
+        <x:v>修正後の修正③</x:v>
+      </x:c>
+      <x:c r="C38" s="19" t="str">
+        <x:v>サーマニードルEVO同意書差し替え、ララドクター詳細・注意事項・副作用の並びと文言、施術不可条件・保護者同意書を更新、料金表削除</x:v>
+      </x:c>
+      <x:c r="D38" s="19" t="str">
+        <x:v>未対応</x:v>
+      </x:c>
+      <x:c r="E38" s="19" t="str">
+        <x:v>対象外</x:v>
+      </x:c>
+      <x:c r="F38" s="19" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="G38" s="19" t="str">
+        <x:v>既存施術ページの文言・構成・添付書類・価格表の修正。</x:v>
+      </x:c>
+      <x:c r="H38" s="19" t="str">
+        <x:v>2026-07-26 受信</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="56" customHeight="1">
+      <x:c r="A39" s="19" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="B39" s="19" t="str">
+        <x:v>修正後の修正④</x:v>
+      </x:c>
+      <x:c r="C39" s="19" t="str">
+        <x:v>美肌治療ページのスマホ表題を短縮・改行調整（サーマニードルEVO、ダーマペン4、KOライト、ララドクター、リバースピール、タトゥー除去、ピコレーザー）</x:v>
+      </x:c>
+      <x:c r="D39" s="19" t="str">
+        <x:v>未対応</x:v>
+      </x:c>
+      <x:c r="E39" s="19" t="str">
+        <x:v>対象外</x:v>
+      </x:c>
+      <x:c r="F39" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G39" s="19" t="str">
+        <x:v>既存ページの表題文言・スマホ表示調整。</x:v>
+      </x:c>
+      <x:c r="H39" s="19" t="str">
+        <x:v>2026-07-26 受信</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="56" customHeight="1">
+      <x:c r="A40" s="19" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="B40" s="19" t="str">
+        <x:v>修正後の修正⑤</x:v>
+      </x:c>
+      <x:c r="C40" s="19" t="str">
+        <x:v>各施術の説明・同意書表記と保護者同意書カード文言を統一</x:v>
+      </x:c>
+      <x:c r="D40" s="19" t="str">
+        <x:v>未対応</x:v>
+      </x:c>
+      <x:c r="E40" s="19" t="str">
+        <x:v>対象外</x:v>
+      </x:c>
+      <x:c r="F40" s="19" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G40" s="19" t="str">
+        <x:v>全施術の既存書類カードの文言修正。</x:v>
+      </x:c>
+      <x:c r="H40" s="19" t="str">
+        <x:v>2026-07-26 受信</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="56" customHeight="1">
+      <x:c r="A41" s="19" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="B41" s="19" t="str">
+        <x:v>修正後の修正⑥</x:v>
+      </x:c>
+      <x:c r="C41" s="19" t="str">
+        <x:v>マッサージピール・リバースピールのホームケア製品名と料金表示をスマホ表示へ調整</x:v>
+      </x:c>
+      <x:c r="D41" s="19" t="str">
+        <x:v>未対応</x:v>
+      </x:c>
+      <x:c r="E41" s="19" t="str">
+        <x:v>対象外</x:v>
+      </x:c>
+      <x:c r="F41" s="19" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G41" s="19" t="str">
+        <x:v>既存施術ページの文言・レスポンシブ表示調整。</x:v>
+      </x:c>
+      <x:c r="H41" s="19" t="str">
+        <x:v>2026-07-26 受信</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="56" customHeight="1">
+      <x:c r="A42" s="19" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+      <x:c r="B42" s="19" t="str">
+        <x:v>修正後の修正⑦</x:v>
+      </x:c>
+      <x:c r="C42" s="19" t="str">
+        <x:v>問診票PDFの不足・ウルティムガン同意書リンク・ララドクターMENU／表題を修正</x:v>
+      </x:c>
+      <x:c r="D42" s="19" t="str">
+        <x:v>一部対応済み／要確認</x:v>
+      </x:c>
+      <x:c r="E42" s="19" t="str">
+        <x:v>対象外</x:v>
+      </x:c>
+      <x:c r="F42" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G42" s="19" t="str">
+        <x:v>既存添付書類導線・MENU・表題の修正。問診票と同意書リンクは対応済みのため、残件を要確認。</x:v>
+      </x:c>
+      <x:c r="H42" s="19" t="str">
+        <x:v>2026-07-27 受信（7/26送信分の追記を含む）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="48" customHeight="1">
+      <x:c r="A43" s="19" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+      <x:c r="B43" s="19" t="str">
+        <x:v>修正後の修正⑧</x:v>
+      </x:c>
+      <x:c r="C43" s="19" t="str">
+        <x:v>ウルティムガン説明・同意書の差し替え、炭酸ガスレーザー問診票の名称変更、価格表の表示順変更・追加麻酔注射削除、ピアモリフティングの修正依頼</x:v>
+      </x:c>
+      <x:c r="D43" s="19" t="str">
+        <x:v>未対応</x:v>
+      </x:c>
+      <x:c r="E43" s="19" t="str">
+        <x:v>対象外</x:v>
+      </x:c>
+      <x:c r="F43" s="19" t="str"/>
+      <x:c r="G43" s="19" t="str">
+        <x:v>添付: ウルティムガン説明・同意書、CO2レーザー問診票。メール本文はピアモリフティングの項目名までで、具体的な修正内容の記載なし。</x:v>
+      </x:c>
+      <x:c r="H43" s="19" t="str">
+        <x:v>メール件名: 修正後の修正⑧（2026-07-27 15:59受信）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>小計</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>見積対象外</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>既存ページ修正、文言差し替え、価格表差し替え、MENU/FAQ削除、注意事項追加、画像・添付差し替え等</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>対象外</x:v>
+      </x:c>
+      <x:c r="F44" t="n">
+        <x:f>SUM(F2:F43)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="G44"/>
+      <x:c r="H44"/>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="R4f4e546d436840aa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="R91f9258cc05248a3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="R29ec796e2e3d4352"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="R4aea723cd0ac44e3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R256522c6fa974fe2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rb60c25c983614bea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="Rd467fa588cee4d74"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="Rab27b031479246c1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="R32ea8896027a4fce"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="R98a09688108c41c6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="Ra9e0ad7c312d4b9b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="R04d5a4aa259a45a0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Rdae956347f924f53"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="R582238b90634435e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R3ed5b94e0e234802"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="R728d65af673947d2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R8cdfbfebd7254061"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="R5caef5a003364e2a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="R494acc041d7b4dfc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="R25ae7e397921415c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="Rdf5b25d241714edd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="R8948ad81e54647bf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="R6eb60fc1d155419a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="R7afa2c26062d49d8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="R223061ab31424661"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="Rdbb6be92395240c4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="R15ad320e6cf3469f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="Rcd1c188cbde94bc6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R287cfc8c099a44ba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="Re7156d781c614d0b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="R18c4cbc952e54be2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R050ae36932384e3c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="R95295066d22c466f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="R4e3875c624144efb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="R21d3106a01114653"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R13b9282f5ba04538"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="Rb6182951caea4a98"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R7a7cd4209c6d4dd4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="R4aea3d8069ba40ad"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="R0164dc196a7f4a63"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="R03dee6570cb44257"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="Rd3d871f9fbd747ee"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2856,590 +3231,688 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="9" t="s">
-        <x:v>208</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="B1" s="9" t="s">
-        <x:v>209</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="C1" s="9" t="s">
-        <x:v>210</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="D1" s="9" t="s">
-        <x:v>211</x:v>
+        <x:v>246</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="5" t="s">
-        <x:v>212</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="B2" s="5" t="s">
-        <x:v>213</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C2" s="5" t="s">
-        <x:v>214</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="D2" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="s">
-        <x:v>216</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="B3" s="5" t="s">
-        <x:v>217</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="C3" s="5" t="s">
-        <x:v>218</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="D3" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="5" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C4" s="5" t="s">
-        <x:v>219</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="D4" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="5" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>38</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>220</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="5" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>221</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="D6" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="5" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>46</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>222</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="D7" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="5" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="s">
+        <x:v>250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="66.25" customHeight="1">
+      <x:c r="A9" s="5" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="37.25" customHeight="1">
-      <x:c r="A9" s="5" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="B9" s="5" t="s">
-        <x:v>55</x:v>
-      </x:c>
       <x:c r="C9" s="5" t="s">
-        <x:v>224</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="D9" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="5" t="s">
-        <x:v>59</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>225</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>226</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="D10" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="5" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B11" s="5" t="s">
-        <x:v>227</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="C11" s="5" t="s">
-        <x:v>228</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="D11" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>229</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="D12" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
-        <x:v>75</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C13" s="5" t="s">
-        <x:v>230</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="D13" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>78</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>79</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D14" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
-        <x:v>81</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C15" s="5" t="s">
-        <x:v>82</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D15" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="5" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B16" s="5" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="C16" s="5" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="C16" s="5" t="s">
-        <x:v>86</x:v>
-      </x:c>
       <x:c r="D16" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="5" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="B17" s="5" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="C17" s="5" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="B17" s="5" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="C17" s="5" t="s">
-        <x:v>118</x:v>
-      </x:c>
       <x:c r="D17" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="5" t="s">
-        <x:v>88</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
-        <x:v>122</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C18" s="5" t="s">
-        <x:v>231</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="D18" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="5" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
-        <x:v>94</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C19" s="5" t="s">
-        <x:v>232</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="D19" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="5" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
-        <x:v>126</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="C20" s="5" t="s">
-        <x:v>233</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="D20" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="5" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B21" s="5" t="s">
-        <x:v>97</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C21" s="5" t="s">
-        <x:v>234</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="D21" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="5" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
-        <x:v>129</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="C22" s="5" t="s">
-        <x:v>235</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="D22" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="5" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="C23" s="5" t="s">
-        <x:v>236</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="D23" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="5" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
-        <x:v>135</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="C24" s="5" t="s">
-        <x:v>237</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="D24" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="5" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C25" s="5" t="s">
-        <x:v>238</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="D25" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B26" s="5" t="s">
-        <x:v>105</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="C26" s="5" t="s">
-        <x:v>239</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="D26" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B27" s="5" t="s">
-        <x:v>138</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="C27" s="5" t="s">
-        <x:v>240</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="D27" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B28" s="5" t="s">
-        <x:v>141</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="C28" s="5" t="s">
-        <x:v>241</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="D28" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B29" s="5" t="s">
-        <x:v>144</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="C29" s="5" t="s">
-        <x:v>242</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="D29" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B30" s="5" t="s">
-        <x:v>147</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="C30" s="5" t="s">
-        <x:v>243</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="D30" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B31" s="5" t="s">
-        <x:v>150</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="C31" s="5" t="s">
-        <x:v>244</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="D31" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B32" s="5" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C32" s="5" t="s">
-        <x:v>245</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="D32" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B33" s="5" t="s">
-        <x:v>155</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C33" s="5" t="s">
-        <x:v>246</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="D33" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="5" t="s">
-        <x:v>108</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B34" s="5" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="C34" s="5" t="s">
-        <x:v>247</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="D34" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="5" t="s">
-        <x:v>108</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B35" s="5" t="s">
-        <x:v>158</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="C35" s="5" t="s">
-        <x:v>248</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D35" s="6" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="20" customHeight="1">
+        <x:v>250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="35.75" customHeight="1">
       <x:c r="A36" s="5" t="s">
-        <x:v>161</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B36" s="5" t="s">
-        <x:v>162</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C36" s="5" t="s">
-        <x:v>249</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="D36" s="14" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="20" customHeight="1">
+        <x:v>250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="35.75" customHeight="1">
       <x:c r="A37" s="5" t="s">
-        <x:v>161</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B37" s="5" t="s">
-        <x:v>165</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="C37" s="5" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="D37" s="14" t="s">
         <x:v>250</x:v>
       </x:c>
-      <x:c r="D37" s="14" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="20" customHeight="1">
+    </x:row>
+    <x:row r="38" ht="35.75" customHeight="1">
       <x:c r="A38" s="5" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B38" s="5" t="s">
-        <x:v>171</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="C38" s="5" t="s">
-        <x:v>251</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="D38" s="14" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="20" customHeight="1">
+        <x:v>250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="35.75" customHeight="1">
       <x:c r="A39" s="5" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B39" s="5" t="s">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="C39" s="5" t="s">
-        <x:v>252</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="D39" s="14" t="s">
-        <x:v>215</x:v>
+        <x:v>250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="B40" t="s">
+        <x:v>236</x:v>
+      </x:c>
+      <x:c r="C40" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="D40" t="s">
+        <x:v>250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="B41" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C41" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="D41" t="s">
+        <x:v>250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>修正後の修正③</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>サーマニードルEVO同意書、ララドクター詳細・料金表・施術不可条件の修正</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>メールを開く</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>修正後の修正④</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>美肌治療ページのスマホ表題を短縮・改行調整</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>メールを開く</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>修正後の修正⑤</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>説明・同意書表記、保護者同意書カード文言の統一</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>メールを開く</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>修正後の修正⑥</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>マッサージピール・リバースピールのホームケア表示調整</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>メールを開く</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>修正後の修正⑦</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>問診票PDF、同意書リンク、ララドクターMENU／表題の修正</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>メールを開く</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="Rce23b6e3a2a04fc0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="R56f5c9770a634dc6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="Rfa3d502e7fb64b68"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="R275db871a72a48a2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="R8c8aaaee37584e00"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="Rc17aaef3a7be4f68"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="Re0de5f6690c34e2e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="R675be7d488ac4276"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="Rffdbf84bef31446e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="Rb46020e5866f4556"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="R3e4bd81637bb4717"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="R85978b73da3a4668"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="Rd8a15597aa574451"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="R1aef7cafa28b45fd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="R65ea922962d0480d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="R38002c0ed6b9470c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="Rc58711555b344c80"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="Rd990e11fb6394889"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="Rcfcea0bb8b2644ff"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="R2eef82bc572b4e21"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="R41fcac35bac84d3c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="R2cda8d46fb6c460f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="R8ab2859a1cd1470d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="Rabb67535c4324ab2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="R17c605390b534ea8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="Re043757f8b3a4bc8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="Ree0185d2496a4073"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="R812f5d3359e844b4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="Re77367fa2f52481c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="R48f4824e2c6647c3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="R324498185bc34a71"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="Rac392ed0878841f4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="R3367389c79ed46b4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="R8b36595247d94bd0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="Rc2b6efbdc4d04fba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="R9d3a8687659741da"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="R23dd20da20c14850"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="R94ac7cc6126045ba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="R5155592705e245c2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="Rf3af91e42fb34901"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R18470af760504b2d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="R0943f9a30dba4dec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="R585b4cad69354a1b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="R9d1b356a760543d1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="R2e01d50437e74d59"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="R40bd62aec41e4bc1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="Rb2144cf7edc347db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="R3e7e17c5d3834af6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="R635d924e67d14b26"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="Rd1c0a2a6cc8a401e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="Rc56933de1f854686"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="Rdf6b6c4552c145d2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="R95d3ce120ddf4e9a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="Ra318fce15ff14c64"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="R48ce631bcd5e4504"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="Re0dad960425f44d5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="Rf52be63597ba47ef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="Rced6b3f3c8df46b3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="R0a635703001d4479"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="R570a27ce75cc4bef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="R9ab2adfbe3884d1b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="Re1bddbff65fb4551"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="Rcd737ca30f724bad"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="Ra3d3e5a81de04693"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="Re92f3538f9ae43bc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="Rb81c42198e054b79"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="R148a96481bcb4773"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="Rfc86c49535a94960"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="R31b6008a7fb14859"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="Ra8b94f5aae9b4fc1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="Rdab6d07ea8184a45"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="Rd5b1ee9aff8e4205"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="R00e12b6069314e82"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="R1ed982d3613a4b1e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="Rbed878b894d84fbd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="R305526fe2e7141c5"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Improve treatment detail layouts and pricing labels
</commit_message>
<xml_diff>
--- a/outputs/mirai-clinic-updates/みらい内科クリニック 美容サイト改修 見積切り分け表.xlsx
+++ b/outputs/mirai-clinic-updates/みらい内科クリニック 美容サイト改修 見積切り分け表.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="1" r:id="R5aa997a062964587"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積対象内" sheetId="2" r:id="Ra3c5e27ba5f34c76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積対象外" sheetId="3" r:id="Rb8a66714405b4a16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メール一覧" sheetId="4" r:id="R74e7f7c406e54b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="1" r:id="R1176f69731834751"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積対象内" sheetId="2" r:id="R104a5950819840b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積対象外" sheetId="3" r:id="Rb8ca782faa8d497f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メール一覧" sheetId="4" r:id="Rfb116d63e3c9426b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37,6 +37,9 @@
     <x:t xml:space="preserve">見積対象外 件数</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">41件（修正後の修正③〜⑦を含む）</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">切り分け基準</x:t>
   </x:si>
   <x:si>
@@ -71,6 +74,9 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">小計値の注意</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Notionの小計行は既存の修正依頼を反映済み。今回、最新メールの「修正後の修正③〜⑦」を追記（⑦は一部対応済み・残件要確認）。</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">備考</x:t>
@@ -549,7 +555,7 @@
   <x:si>
     <x:r>
       <x:rPr>
-        <x:sz val="1000"/>
+        <x:sz val="409"/>
         <x:color rgb="FF1155CC"/>
         <x:rFont val="MS Gothic"/>
         <x:family val="2"/>
@@ -558,7 +564,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1000"/>
+        <x:sz val="409"/>
         <x:color rgb="FF1155CC"/>
         <x:rFont val="Arial"/>
       </x:rPr>
@@ -776,6 +782,81 @@
     <x:t xml:space="preserve">既存ページの表示・書体・文言・価格表・書類カード・FAQの統一。新規サービス追加は含まれない。</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">2026-07-26</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">修正後の修正③</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">サーマニードルEVO同意書差し替え、ララドクター詳細・注意事項・副作用の並びと文言、施術不可条件・保護者同意書を更新、料金表削除</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">既存施術ページの文言・構成・添付書類・価格表の修正。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">2026-07-26 受信</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">修正後の修正④</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美肌治療ページのスマホ表題を短縮・改行調整（サーマニードルEVO、ダーマペン4、KOライト、ララドクター、リバースピール、タトゥー除去、ピコレーザー）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">既存ページの表題文言・スマホ表示調整。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">修正後の修正⑤</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">各施術の説明・同意書表記と保護者同意書カード文言を統一</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">全施術の既存書類カードの文言修正。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">修正後の修正⑥</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">マッサージピール・リバースピールのホームケア製品名と料金表示をスマホ表示へ調整</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">既存施術ページの文言・レスポンシブ表示調整。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">2026-07-27</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">修正後の修正⑦</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">問診票PDFの不足・ウルティムガン同意書リンク・ララドクターMENU／表題を修正</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">既存添付書類導線・MENU・表題の修正。問診票と同意書リンクは対応済みのため、残件を要確認。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">2026-07-27 受信（7/26送信分の追記を含む）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">修正後の修正⑧</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">ウルティムガン説明・同意書の差し替え、炭酸ガスレーザー問診票の名称変更、価格表の表示順変更・追加麻酔注射削除、ピアモリフティングの修正依頼</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">添付: ウルティムガン説明・同意書、CO2レーザー問診票。メール本文はピアモリフティングの項目名までで、具体的な修正内容の記載なし。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">メール件名: 修正後の修正⑧（2026-07-27 15:59受信）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">見積対象外</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">既存ページ修正、文言差し替え、価格表差し替え、MENU/FAQ削除、注意事項追加、画像・添付差し替え等</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">日付</x:t>
   </x:si>
   <x:si>
@@ -915,13 +996,28 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CO2・共通価格表・書類カード・保護者同意書・FAQの修正</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">サーマニードルEVO同意書、ララドクター詳細・料金表・施術不可条件の修正</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美肌治療ページのスマホ表題を短縮・改行調整</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">説明・同意書表記、保護者同意書カード文言の統一</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">マッサージピール・リバースピールのホームケア表示調整</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">問診票PDF、同意書リンク、ララドクターMENU／表題の修正</x:t>
   </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="18">
+  <x:fonts count="19">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -986,6 +1082,21 @@
       <x:name val="Arial"/>
     </x:font>
     <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1155CC"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="409"/>
+      <x:color rgb="FF1155CC"/>
+      <x:name val="MS Gothic"/>
+    </x:font>
+    <x:font>
+      <x:sz val="409"/>
+      <x:color rgb="FF1155CC"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
       <x:sz val="409"/>
       <x:color rgb="FF1155CC"/>
       <x:name val="MS Gothic"/>
@@ -998,16 +1109,6 @@
     <x:font>
       <x:sz val="6"/>
       <x:name val="07NikumaruFont"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF1155CC"/>
-      <x:name val="MS Gothic"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF1155CC"/>
-      <x:name val="Arial"/>
     </x:font>
   </x:fonts>
   <x:fills count="6">
@@ -1106,14 +1207,14 @@
     <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -1343,7 +1444,7 @@
     <x:col min="2" max="2" width="80" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="42.75" customHeight="1">
+    <x:row r="1" ht="57" customHeight="1">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -1380,8 +1481,8 @@
       <x:c r="A6" s="2" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B6" s="3" t="str">
-        <x:v>41件（修正後の修正③〜⑦を含む）</x:v>
+      <x:c r="B6" s="3" t="s">
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1390,64 +1491,64 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B8" s="3"/>
     </x:row>
-    <x:row r="9" ht="66.25" customHeight="1">
+    <x:row r="9" ht="88.25" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="66.25" customHeight="1">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="88.25" customHeight="1">
       <x:c r="A10" s="2" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
-        <x:v>12</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="66.25" customHeight="1">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="88.25" customHeight="1">
       <x:c r="A11" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="66.25" customHeight="1">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="88.25" customHeight="1">
       <x:c r="A12" s="2" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="66.25" customHeight="1">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="88.25" customHeight="1">
       <x:c r="A13" s="2" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
-        <x:v>18</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="66.25" customHeight="1">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="88.25" customHeight="1">
       <x:c r="A14" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B14" s="20" t="str">
-        <x:v>Notionの小計行は既存の修正依頼を反映済み。今回、最新メールの「修正後の修正③〜⑦」を追記（⑦は一部対応済み・残件要確認）。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="66.25" customHeight="1">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="s">
+        <x:v>21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="88.25" customHeight="1">
       <x:c r="A15" s="2" t="s">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1469,541 +1570,541 @@
     <x:col min="8" max="8" width="26" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="35.75" customHeight="1">
+    <x:row r="1" ht="47.75" customHeight="1">
       <x:c r="A1" s="4" t="s">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B1" s="4" t="s">
-        <x:v>23</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C1" s="4" t="s">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D1" s="4" t="s">
-        <x:v>25</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E1" s="4" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F1" s="13" t="s">
-        <x:v>27</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="G1" s="4" t="s">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="H1" s="4" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="66.25" customHeight="1">
+        <x:v>31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="88.25" customHeight="1">
       <x:c r="A2" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B2" s="5" t="s">
-        <x:v>31</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C2" s="5" t="s">
-        <x:v>32</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D2" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E2" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F2" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G2" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="H2" s="6" t="s">
-        <x:v>31</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="66.25" customHeight="1">
+        <x:v>33</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="88.25" customHeight="1">
       <x:c r="A3" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B3" s="5" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C3" s="5" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D3" s="5" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E3" s="5" t="s">
         <x:v>36</x:v>
-      </x:c>
-      <x:c r="C3" s="5" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D3" s="5" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E3" s="5" t="s">
-        <x:v>34</x:v>
       </x:c>
       <x:c r="F3" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G3" s="5" t="s">
-        <x:v>39</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="H3" s="6" t="s">
+        <x:v>38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="88.25" customHeight="1">
+      <x:c r="A4" s="5" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="s">
         <x:v>36</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="66.25" customHeight="1">
-      <x:c r="A4" s="5" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E4" s="5" t="s">
-        <x:v>34</x:v>
       </x:c>
       <x:c r="F4" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G4" s="5" t="s">
-        <x:v>43</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="H4" s="6" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>44</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>45</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F5" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="5" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="H5" s="6" t="s">
-        <x:v>44</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="6" ht="88.25" customHeight="1">
       <x:c r="A6" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>47</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
-        <x:v>49</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F6" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="5" t="s">
-        <x:v>50</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="H6" s="6" t="s">
-        <x:v>51</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="66.25" customHeight="1">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="88.25" customHeight="1">
       <x:c r="A7" s="5" t="s">
-        <x:v>52</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
-        <x:v>55</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E7" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F7" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G7" s="5" t="s">
-        <x:v>56</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="H7" s="6" t="s">
-        <x:v>53</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="66.25" customHeight="1">
+        <x:v>55</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="88.25" customHeight="1">
       <x:c r="A8" s="5" t="s">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>58</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>59</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D8" s="5" t="s">
-        <x:v>60</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F8" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G8" s="5" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="H8" s="6" t="s">
-        <x:v>62</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="66.25" customHeight="1">
+        <x:v>64</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="88.25" customHeight="1">
       <x:c r="A9" s="5" t="s">
-        <x:v>63</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B9" s="5" t="s">
-        <x:v>64</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C9" s="5" t="s">
-        <x:v>65</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D9" s="5" t="s">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F9" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="5" t="s">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="H9" s="6" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>70</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F10" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="5" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="s">
         <x:v>72</x:v>
-      </x:c>
-      <x:c r="H10" s="6" t="s">
-        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B11" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C11" s="5" t="s">
-        <x:v>74</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D11" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F11" s="10">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G11" s="5" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="s">
         <x:v>75</x:v>
-      </x:c>
-      <x:c r="H11" s="6" t="s">
-        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D12" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F12" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G12" s="5" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="H12" s="6" t="s">
-        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
-        <x:v>79</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C13" s="5" t="s">
-        <x:v>80</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D13" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F13" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="5" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="s">
         <x:v>81</x:v>
-      </x:c>
-      <x:c r="H13" s="6" t="s">
-        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="5" t="s">
-        <x:v>82</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>83</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>84</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="D14" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F14" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G14" s="5" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="H14" s="6" t="s">
-        <x:v>83</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="15" ht="88.25" customHeight="1">
       <x:c r="A15" s="5" t="s">
-        <x:v>86</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
-        <x:v>87</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C15" s="5" t="s">
-        <x:v>88</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D15" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E15" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F15" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G15" s="5" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="H15" s="6" t="s">
-        <x:v>90</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="66.25" customHeight="1">
+        <x:v>92</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="88.25" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
-        <x:v>92</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
-        <x:v>93</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="D16" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F16" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G16" s="5" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="H16" s="6" t="s">
-        <x:v>92</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="17" ht="88.25" customHeight="1">
       <x:c r="A17" s="5" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B17" s="5" t="s">
-        <x:v>95</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C17" s="5" t="s">
-        <x:v>96</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D17" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E17" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F17" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G17" s="5" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="H17" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="H17" s="6" t="s">
-        <x:v>95</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="18" ht="88.25" customHeight="1">
       <x:c r="A18" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
-        <x:v>99</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C18" s="5" t="s">
-        <x:v>100</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D18" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E18" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F18" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G18" s="5" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="H18" s="6" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="H18" s="6" t="s">
-        <x:v>99</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="99.75" customHeight="1">
+    </x:row>
+    <x:row r="19" ht="133" customHeight="1">
       <x:c r="A19" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
-        <x:v>103</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C19" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D19" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E19" s="12" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F19" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="5" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="H19" s="6" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="H19" s="6" t="s">
-        <x:v>103</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="99.75" customHeight="1">
+    </x:row>
+    <x:row r="20" ht="133" customHeight="1">
       <x:c r="A20" s="5" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
-        <x:v>107</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C20" s="5" t="s">
-        <x:v>108</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="D20" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E20" s="12" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F20" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G20" s="5" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="H20" s="6" t="s">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="H20" s="6" t="s">
-        <x:v>107</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="21" ht="88.25" customHeight="1">
       <x:c r="A21" s="7" t="s">
-        <x:v>110</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B21" s="7" t="s">
-        <x:v>111</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C21" s="7" t="s">
-        <x:v>112</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="D21" s="7" t="s">
-        <x:v>113</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="E21" s="7" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F21" s="7" t="n">
         <x:f>SUM(F2:F20)</x:f>
@@ -2014,25 +2115,25 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="R4d4bb2da9b1c4228"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="Ra9e1dddd3ecc48f6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="R6231fd0a4d9045b3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="Rca791d064a44464c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R0a5ab329a9694c1f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rc18e353e40d84316"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="R7534dcb02ef94ab8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R05c65a96865b462b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="Rc02b69d857344427"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="Rf30e7d35b136425a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R6a2d3ec3be1a44f1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="R98dc4b6b632d4e17"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Red81e1b966344068"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="Rcaaded9020be4d78"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="Ref1bd6d1220543ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="Ra44f0391cca040c9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="Re92130abeb1d4934"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="R573a4caa513149b2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R772b86e931a34c35"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="Rf0310ec97c0547bb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="R0908b80c678b4aa3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="R96731bfd113449ac"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="R3fa67fef9d154b68"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R1bd696c31caf494f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rf9eb3c3cd9444da3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="R1d52d6f20aa343b4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R1cf62f7f445c402c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="R6be711a315184307"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="Rd181772f5d2f4baa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R70ffcdc74993422e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="Rbf37b7a71dc84006"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="R7545a95a75a14fb5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="R390c0bbd90b143e1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="R50920e7f6f0b4f8e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="R0ba10a58996f401e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="Rd1958de7450a4e49"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="R6ea63e2f71d344f8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="Rea6278b9d8ae463e"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2052,1168 +2153,1266 @@
     <x:col min="8" max="8" width="26" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="35.75" customHeight="1">
+    <x:row r="1" ht="47.75" customHeight="1">
       <x:c r="A1" s="8" t="s">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B1" s="8" t="s">
-        <x:v>23</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C1" s="8" t="s">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D1" s="8" t="s">
-        <x:v>25</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E1" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F1" s="11" t="s">
-        <x:v>27</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="G1" s="8" t="s">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="H1" s="8" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="99.75" customHeight="1">
+        <x:v>31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="133" customHeight="1">
       <x:c r="A2" s="5" t="s">
-        <x:v>114</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B2" s="5" t="s">
-        <x:v>115</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C2" s="5" t="s">
-        <x:v>116</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="D2" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E2" s="12" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F2" s="10">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G2" s="5" t="s">
-        <x:v>118</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="H2" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="66.25" customHeight="1">
+        <x:v>117</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="88.25" customHeight="1">
       <x:c r="A3" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B3" s="5" t="s">
-        <x:v>120</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="C3" s="5" t="s">
-        <x:v>121</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="D3" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E3" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F3" s="10">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G3" s="5" t="s">
-        <x:v>122</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="H3" s="6" t="s">
-        <x:v>123</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="133" customHeight="1">
+        <x:v>125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="177.25" customHeight="1">
       <x:c r="A4" s="5" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>124</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C4" s="5" t="s">
-        <x:v>125</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F4" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G4" s="5" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="H4" s="6" t="s">
-        <x:v>124</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="5" ht="88.25" customHeight="1">
       <x:c r="A5" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>127</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>128</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D5" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F5" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G5" s="5" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="H5" s="6" t="s">
-        <x:v>127</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="6" ht="88.25" customHeight="1">
       <x:c r="A6" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>131</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D6" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F6" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G6" s="5" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="H6" s="6" t="s">
-        <x:v>130</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="35.75" customHeight="1">
+    </x:row>
+    <x:row r="7" ht="47.75" customHeight="1">
       <x:c r="A7" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>133</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>134</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D7" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E7" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F7" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G7" s="5" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="s">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="H7" s="6" t="s">
-        <x:v>133</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="8" ht="88.25" customHeight="1">
       <x:c r="A8" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>136</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>137</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="D8" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F8" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G8" s="5" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="H8" s="6" t="s">
-        <x:v>136</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="9" ht="88.25" customHeight="1">
       <x:c r="A9" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B9" s="5" t="s">
-        <x:v>139</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C9" s="5" t="s">
-        <x:v>140</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="D9" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F9" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G9" s="5" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="H9" s="6" t="s">
-        <x:v>139</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="35.75" customHeight="1">
+    </x:row>
+    <x:row r="10" ht="47.75" customHeight="1">
       <x:c r="A10" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>142</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>143</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="D10" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F10" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G10" s="5" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="s">
         <x:v>144</x:v>
       </x:c>
-      <x:c r="H10" s="6" t="s">
-        <x:v>142</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="11" ht="88.25" customHeight="1">
       <x:c r="A11" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B11" s="5" t="s">
-        <x:v>145</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C11" s="5" t="s">
-        <x:v>146</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="D11" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F11" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G11" s="5" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="H11" s="6" t="s">
-        <x:v>145</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="12" ht="88.25" customHeight="1">
       <x:c r="A12" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>148</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>149</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="D12" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F12" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G12" s="5" t="s">
-        <x:v>147</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="H12" s="6" t="s">
-        <x:v>148</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="66.25" customHeight="1">
+        <x:v>150</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="88.25" customHeight="1">
       <x:c r="A13" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
-        <x:v>150</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="C13" s="5" t="s">
-        <x:v>151</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="D13" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F13" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G13" s="5" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="s">
         <x:v>152</x:v>
       </x:c>
-      <x:c r="H13" s="6" t="s">
-        <x:v>150</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="99.75" customHeight="1">
+    </x:row>
+    <x:row r="14" ht="133" customHeight="1">
       <x:c r="A14" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>153</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>154</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D14" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F14" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G14" s="5" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="H14" s="6" t="s">
-        <x:v>153</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="15" ht="88.25" customHeight="1">
       <x:c r="A15" s="5" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
-        <x:v>156</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="C15" s="5" t="s">
-        <x:v>157</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="D15" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E15" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F15" s="5">
         <x:v>3</x:v>
       </x:c>
       <x:c r="G15" s="5" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="H15" s="6" t="s">
         <x:v>158</x:v>
       </x:c>
-      <x:c r="H15" s="6" t="s">
-        <x:v>156</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="99.75" customHeight="1">
+    </x:row>
+    <x:row r="16" ht="133" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>159</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
-        <x:v>160</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
-        <x:v>161</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="D16" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F16" s="5">
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="G16" s="5" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="s">
         <x:v>162</x:v>
       </x:c>
-      <x:c r="H16" s="6" t="s">
-        <x:v>160</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="66.25" customHeight="1">
+    </x:row>
+    <x:row r="17" ht="88.25" customHeight="1">
       <x:c r="A17" s="5" t="s">
-        <x:v>159</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B17" s="5" t="s">
-        <x:v>163</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="C17" s="5" t="s">
-        <x:v>164</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="D17" s="5" t="s">
-        <x:v>165</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="E17" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F17" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G17" s="5" t="s">
-        <x:v>166</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="H17" s="16" t="s">
-        <x:v>167</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="66.25" customHeight="1">
+        <x:v>169</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="88.25" customHeight="1">
       <x:c r="A18" s="5" t="s">
-        <x:v>168</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
-        <x:v>169</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="C18" s="5" t="s">
-        <x:v>170</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="D18" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E18" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F18" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G18" s="5" t="s">
-        <x:v>171</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="H18" s="18" t="s">
-        <x:v>172</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="66.25" customHeight="1">
+        <x:v>174</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="88.25" customHeight="1">
       <x:c r="A19" s="5" t="s">
-        <x:v>168</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
-        <x:v>173</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="C19" s="5" t="s">
-        <x:v>174</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="D19" s="12" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E19" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F19" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="5" t="s">
-        <x:v>175</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="H19" s="6" t="s">
-        <x:v>176</x:v>
+        <x:v>178</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28">
       <x:c r="A20" s="5" t="s">
-        <x:v>177</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
-        <x:v>178</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C20" s="5" t="s">
-        <x:v>179</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="D20" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E20" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F20" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G20" s="5" t="s">
-        <x:v>180</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="H20" s="15" t="s">
-        <x:v>181</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="28">
       <x:c r="A21" s="5" t="s">
-        <x:v>177</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B21" s="5" t="s">
-        <x:v>182</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C21" s="5" t="s">
-        <x:v>183</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="D21" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E21" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F21" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G21" s="5" t="s">
-        <x:v>184</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="H21" s="15" t="s">
-        <x:v>185</x:v>
+        <x:v>187</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28">
       <x:c r="A22" s="5" t="s">
-        <x:v>177</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
-        <x:v>186</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="C22" s="5" t="s">
-        <x:v>187</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="D22" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E22" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F22" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G22" s="5" t="s">
-        <x:v>188</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="H22" s="15" t="s">
-        <x:v>189</x:v>
+        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42">
       <x:c r="A23" s="5" t="s">
-        <x:v>177</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
-        <x:v>190</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="C23" s="5" t="s">
-        <x:v>191</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="D23" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E23" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F23" s="5">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G23" s="5" t="s">
-        <x:v>192</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="H23" s="15" t="s">
-        <x:v>193</x:v>
+        <x:v>195</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42">
       <x:c r="A24" s="5" t="s">
-        <x:v>177</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
-        <x:v>194</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="C24" s="5" t="s">
-        <x:v>195</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="D24" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E24" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F24" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G24" s="5" t="s">
-        <x:v>196</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="H24" s="15" t="s">
-        <x:v>197</x:v>
+        <x:v>199</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42">
       <x:c r="A25" s="5" t="s">
-        <x:v>177</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
-        <x:v>198</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="C25" s="5" t="s">
-        <x:v>199</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="D25" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E25" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F25" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G25" s="5" t="s">
-        <x:v>200</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="H25" s="15" t="s">
-        <x:v>201</x:v>
+        <x:v>203</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28">
       <x:c r="A26" s="5" t="s">
-        <x:v>202</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="B26" s="5" t="s">
-        <x:v>203</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="C26" s="5" t="s">
-        <x:v>204</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D26" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E26" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F26" s="5">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G26" s="5" t="s">
-        <x:v>205</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="H26" s="15" t="s">
-        <x:v>206</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="53.25" customHeight="1">
+        <x:v>208</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="71" customHeight="1">
       <x:c r="A27" t="s">
-        <x:v>207</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B27" t="s">
-        <x:v>208</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="C27" t="s">
-        <x:v>209</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="D27" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E27" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F27">
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="G27" t="s">
-        <x:v>210</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="H27" t="s">
-        <x:v>211</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="29.25" customHeight="1">
+        <x:v>213</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="39" customHeight="1">
       <x:c r="A28" t="s">
-        <x:v>207</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B28" t="s">
-        <x:v>212</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="C28" t="s">
-        <x:v>213</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="D28" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E28" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F28" s="17">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G28" t="s">
-        <x:v>214</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="H28" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="36" customHeight="1">
+        <x:v>217</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="48" customHeight="1">
       <x:c r="A29" t="s">
-        <x:v>207</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B29" t="s">
-        <x:v>216</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C29" t="s">
-        <x:v>217</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="D29" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E29" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F29" s="17">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G29" t="s">
-        <x:v>218</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="H29" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="40" customHeight="1">
+        <x:v>217</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="53.25" customHeight="1">
       <x:c r="A30" t="s">
-        <x:v>207</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B30" t="s">
-        <x:v>219</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="C30" t="s">
-        <x:v>220</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="D30" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E30" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F30" s="17">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G30" t="s">
-        <x:v>221</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="H30" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="36" customHeight="1">
+        <x:v>217</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="48" customHeight="1">
       <x:c r="A31" t="s">
-        <x:v>207</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B31" t="s">
-        <x:v>222</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="C31" t="s">
-        <x:v>223</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="D31" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E31" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F31" s="17">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" t="s">
-        <x:v>224</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="H31" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="33.25" customHeight="1">
+        <x:v>217</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="44.25" customHeight="1">
       <x:c r="A32" t="s">
-        <x:v>207</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B32" t="s">
-        <x:v>225</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="C32" t="s">
-        <x:v>226</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="D32" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E32" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F32" s="17">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G32" t="s">
-        <x:v>227</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="H32" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="36" customHeight="1">
+        <x:v>217</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="48" customHeight="1">
       <x:c r="A33" t="s">
-        <x:v>207</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B33" t="s">
-        <x:v>228</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C33" t="s">
-        <x:v>229</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="D33" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E33" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F33" s="17">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G33" t="s">
-        <x:v>230</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="H33" t="s">
-        <x:v>215</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="20" customHeight="1">
+        <x:v>217</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="26.75" customHeight="1">
       <x:c r="A34" t="s">
-        <x:v>207</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B34" t="s">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c r="C34" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="C34" t="s">
-        <x:v>229</x:v>
-      </x:c>
       <x:c r="D34" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E34" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F34" s="17">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G34" t="s">
-        <x:v>232</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="H34" t="s">
-        <x:v>215</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="s">
-        <x:v>207</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B35" t="s">
-        <x:v>233</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C35" t="s">
-        <x:v>229</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="D35" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E35" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F35" s="17">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G35" t="s">
-        <x:v>234</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="H35" t="s">
-        <x:v>215</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="s">
-        <x:v>235</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="B36" t="s">
-        <x:v>236</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="C36" t="s">
-        <x:v>237</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D36" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E36" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F36">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G36" t="s">
-        <x:v>238</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H36" t="s">
-        <x:v>239</x:v>
+        <x:v>241</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="s">
-        <x:v>235</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="B37" t="s">
-        <x:v>240</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="C37" t="s">
-        <x:v>241</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="D37" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E37" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F37">
         <x:v>3.5</x:v>
       </x:c>
       <x:c r="G37" t="s">
-        <x:v>242</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="H37" t="s">
-        <x:v>239</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="56" customHeight="1">
-      <x:c r="A38" s="19" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="B38" s="19" t="str">
-        <x:v>修正後の修正③</x:v>
-      </x:c>
-      <x:c r="C38" s="19" t="str">
-        <x:v>サーマニードルEVO同意書差し替え、ララドクター詳細・注意事項・副作用の並びと文言、施術不可条件・保護者同意書を更新、料金表削除</x:v>
-      </x:c>
-      <x:c r="D38" s="19" t="str">
+        <x:v>241</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="74.75" customHeight="1">
+      <x:c r="A38" s="19" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="B38" s="19" t="s">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="C38" s="19" t="s">
+        <x:v>247</x:v>
+      </x:c>
+      <x:c r="D38" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="E38" s="19" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="F38" s="19">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G38" s="19" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="H38" s="19" t="s">
+        <x:v>249</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="74.75" customHeight="1">
+      <x:c r="A39" s="19" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="B39" s="19" t="s">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="C39" s="19" t="s">
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="D39" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="E39" s="19" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="F39" s="19">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G39" s="19" t="s">
+        <x:v>252</x:v>
+      </x:c>
+      <x:c r="H39" s="19" t="s">
+        <x:v>249</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="74.75" customHeight="1">
+      <x:c r="A40" s="19" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="B40" s="19" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="C40" s="19" t="s">
+        <x:v>254</x:v>
+      </x:c>
+      <x:c r="D40" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="E40" s="19" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="F40" s="19">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G40" s="19" t="s">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="H40" s="19" t="s">
+        <x:v>249</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="74.75" customHeight="1">
+      <x:c r="A41" s="19" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="B41" s="19" t="s">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C41" s="19" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="D41" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="E41" s="19" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="F41" s="19">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G41" s="19" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="H41" s="19" t="s">
+        <x:v>249</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="74.75" customHeight="1">
+      <x:c r="A42" s="19" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="B42" s="19" t="s">
+        <x:v>260</x:v>
+      </x:c>
+      <x:c r="C42" s="19" t="s">
+        <x:v>261</x:v>
+      </x:c>
+      <x:c r="D42" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="E42" s="19" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="F42" s="19">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G42" s="19" t="s">
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="H42" s="19" t="s">
+        <x:v>263</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="64" customHeight="1">
+      <x:c r="A43" s="19" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="B43" s="19" t="s">
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="C43" s="19" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="D43" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="E43" s="19" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="F43" s="19">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G43" s="19" t="s">
+        <x:v>266</x:v>
+      </x:c>
+      <x:c r="H43" s="19" t="s">
+        <x:v>267</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="84" customHeight="1">
+      <x:c r="A44" s="20" t="str">
+        <x:v>2026-07-28</x:v>
+      </x:c>
+      <x:c r="B44" s="20" t="str">
+        <x:v>修正後の修正⑧ 追加対応</x:v>
+      </x:c>
+      <x:c r="C44" s="20" t="str">
+        <x:v>炭酸ガスレーザー問診票リンク差し替え、美肌治療価格表の炭酸ガスレーザー表記変更・追加麻酔注射削除、ピアモリフティングのボディ表記・スマホ行頭調整、共通20ページへ反映</x:v>
+      </x:c>
+      <x:c r="D44" s="20" t="str">
+        <x:v>対応済み</x:v>
+      </x:c>
+      <x:c r="E44" s="20" t="str">
+        <x:v>対象外</x:v>
+      </x:c>
+      <x:c r="F44" s="20" t="str"/>
+      <x:c r="G44" s="20" t="str">
+        <x:v>既存ページ・共通価格表のリンク、文言、レスポンシブ表示を修正。新規サービス追加は含まれない。</x:v>
+      </x:c>
+      <x:c r="H44" s="20" t="str">
+        <x:v>チャット依頼（2026-07-27～2026-07-28）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="84" customHeight="1">
+      <x:c r="A45" s="20" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+      <x:c r="B45" s="20" t="str">
+        <x:v>修正後の修正⑨</x:v>
+      </x:c>
+      <x:c r="C45" s="20" t="str">
+        <x:v>ダーマペン4のセクション間隔・表示順変更、施術不可条件のPC／スマホ改行調整。ピアモリフティングの対象部位表記を「ボディー」から「ボディ」へ変更</x:v>
+      </x:c>
+      <x:c r="D45" s="20" t="str">
         <x:v>未対応</x:v>
       </x:c>
-      <x:c r="E38" s="19" t="str">
+      <x:c r="E45" s="20" t="str">
         <x:v>対象外</x:v>
       </x:c>
-      <x:c r="F38" s="19" t="n">
-        <x:v>2.5</x:v>
-      </x:c>
-      <x:c r="G38" s="19" t="str">
-        <x:v>既存施術ページの文言・構成・添付書類・価格表の修正。</x:v>
-      </x:c>
-      <x:c r="H38" s="19" t="str">
-        <x:v>2026-07-26 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="56" customHeight="1">
-      <x:c r="A39" s="19" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="B39" s="19" t="str">
-        <x:v>修正後の修正④</x:v>
-      </x:c>
-      <x:c r="C39" s="19" t="str">
-        <x:v>美肌治療ページのスマホ表題を短縮・改行調整（サーマニードルEVO、ダーマペン4、KOライト、ララドクター、リバースピール、タトゥー除去、ピコレーザー）</x:v>
-      </x:c>
-      <x:c r="D39" s="19" t="str">
+      <x:c r="F45" s="20" t="str"/>
+      <x:c r="G45" s="20" t="str">
+        <x:v>既存ページの構成・文言・レスポンシブ改行調整。添付画像4点による表示指示を含む。</x:v>
+      </x:c>
+      <x:c r="H45" s="20" t="str">
+        <x:v>メール件名: 修正後の修正⑨（2026-07-27 23:49受信）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="84" customHeight="1">
+      <x:c r="A46" s="20" t="str">
+        <x:v>2026-07-28</x:v>
+      </x:c>
+      <x:c r="B46" s="20" t="str">
+        <x:v>修正後の修正⑩（タトゥー除去・レーザーフェイシャル）</x:v>
+      </x:c>
+      <x:c r="C46" s="20" t="str">
+        <x:v>タトゥー除去の施術不可条件へ10項目を赤文字で追加。レーザーフェイシャルの注意事項を「メイクは施術翌日から可能」から「施術当日から可能」へ変更</x:v>
+      </x:c>
+      <x:c r="D46" s="20" t="str">
         <x:v>未対応</x:v>
       </x:c>
-      <x:c r="E39" s="19" t="str">
+      <x:c r="E46" s="20" t="str">
         <x:v>対象外</x:v>
       </x:c>
-      <x:c r="F39" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G39" s="19" t="str">
-        <x:v>既存ページの表題文言・スマホ表示調整。</x:v>
-      </x:c>
-      <x:c r="H39" s="19" t="str">
-        <x:v>2026-07-26 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="56" customHeight="1">
-      <x:c r="A40" s="19" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="B40" s="19" t="str">
-        <x:v>修正後の修正⑤</x:v>
-      </x:c>
-      <x:c r="C40" s="19" t="str">
-        <x:v>各施術の説明・同意書表記と保護者同意書カード文言を統一</x:v>
-      </x:c>
-      <x:c r="D40" s="19" t="str">
+      <x:c r="F46" s="20" t="str"/>
+      <x:c r="G46" s="20" t="str">
+        <x:v>既存ページの施術不可条件・注意事項の追記および文言変更。添付画像2点を含む。</x:v>
+      </x:c>
+      <x:c r="H46" s="20" t="str">
+        <x:v>メール件名: 修正後の修正⑩（2026-07-28 00:03受信）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="84" customHeight="1">
+      <x:c r="A47" s="20" t="str">
+        <x:v>2026-07-28</x:v>
+      </x:c>
+      <x:c r="B47" s="20" t="str">
+        <x:v>修正後の修正⑩（価格表スマホ表示）</x:v>
+      </x:c>
+      <x:c r="C47" s="20" t="str">
+        <x:v>美肌治療価格表すべてについて、スマホ縦・横画面の右側余白を減らし、施術内容を左・価格を右に配置。施術内容の2段表示や文字サイズ調整も含めて見やすくする</x:v>
+      </x:c>
+      <x:c r="D47" s="20" t="str">
         <x:v>未対応</x:v>
       </x:c>
-      <x:c r="E40" s="19" t="str">
+      <x:c r="E47" s="20" t="str">
         <x:v>対象外</x:v>
       </x:c>
-      <x:c r="F40" s="19" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="G40" s="19" t="str">
-        <x:v>全施術の既存書類カードの文言修正。</x:v>
-      </x:c>
-      <x:c r="H40" s="19" t="str">
-        <x:v>2026-07-26 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="56" customHeight="1">
-      <x:c r="A41" s="19" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="B41" s="19" t="str">
-        <x:v>修正後の修正⑥</x:v>
-      </x:c>
-      <x:c r="C41" s="19" t="str">
-        <x:v>マッサージピール・リバースピールのホームケア製品名と料金表示をスマホ表示へ調整</x:v>
-      </x:c>
-      <x:c r="D41" s="19" t="str">
-        <x:v>未対応</x:v>
-      </x:c>
-      <x:c r="E41" s="19" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F41" s="19" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="G41" s="19" t="str">
-        <x:v>既存施術ページの文言・レスポンシブ表示調整。</x:v>
-      </x:c>
-      <x:c r="H41" s="19" t="str">
-        <x:v>2026-07-26 受信</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="56" customHeight="1">
-      <x:c r="A42" s="19" t="str">
-        <x:v>2026-07-27</x:v>
-      </x:c>
-      <x:c r="B42" s="19" t="str">
-        <x:v>修正後の修正⑦</x:v>
-      </x:c>
-      <x:c r="C42" s="19" t="str">
-        <x:v>問診票PDFの不足・ウルティムガン同意書リンク・ララドクターMENU／表題を修正</x:v>
-      </x:c>
-      <x:c r="D42" s="19" t="str">
-        <x:v>一部対応済み／要確認</x:v>
-      </x:c>
-      <x:c r="E42" s="19" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F42" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G42" s="19" t="str">
-        <x:v>既存添付書類導線・MENU・表題の修正。問診票と同意書リンクは対応済みのため、残件を要確認。</x:v>
-      </x:c>
-      <x:c r="H42" s="19" t="str">
-        <x:v>2026-07-27 受信（7/26送信分の追記を含む）</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="48" customHeight="1">
-      <x:c r="A43" s="19" t="str">
-        <x:v>2026-07-27</x:v>
-      </x:c>
-      <x:c r="B43" s="19" t="str">
-        <x:v>修正後の修正⑧</x:v>
-      </x:c>
-      <x:c r="C43" s="19" t="str">
-        <x:v>ウルティムガン説明・同意書の差し替え、炭酸ガスレーザー問診票の名称変更、価格表の表示順変更・追加麻酔注射削除、ピアモリフティングの修正依頼</x:v>
-      </x:c>
-      <x:c r="D43" s="19" t="str">
-        <x:v>未対応</x:v>
-      </x:c>
-      <x:c r="E43" s="19" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F43" s="19" t="str"/>
-      <x:c r="G43" s="19" t="str">
-        <x:v>添付: ウルティムガン説明・同意書、CO2レーザー問診票。メール本文はピアモリフティングの項目名までで、具体的な修正内容の記載なし。</x:v>
-      </x:c>
-      <x:c r="H43" s="19" t="str">
-        <x:v>メール件名: 修正後の修正⑧（2026-07-27 15:59受信）</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" t="str">
-        <x:v>小計</x:v>
-      </x:c>
-      <x:c r="B44" t="str">
-        <x:v>見積対象外</x:v>
-      </x:c>
-      <x:c r="C44" t="str">
-        <x:v>既存ページ修正、文言差し替え、価格表差し替え、MENU/FAQ削除、注意事項追加、画像・添付差し替え等</x:v>
-      </x:c>
-      <x:c r="D44" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="E44" t="str">
-        <x:v>対象外</x:v>
-      </x:c>
-      <x:c r="F44" t="n">
-        <x:f>SUM(F2:F43)</x:f>
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="G44"/>
-      <x:c r="H44"/>
+      <x:c r="F47" s="20" t="str"/>
+      <x:c r="G47" s="20" t="str">
+        <x:v>6/27美容修正P2の追加調整。既存の共通価格表に対するレスポンシブ表示改善。添付画像3点を含む。</x:v>
+      </x:c>
+      <x:c r="H47" s="20" t="str">
+        <x:v>メール件名: 修正後の修正⑩（2026-07-28 08:48受信）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="B48" t="s">
+        <x:v>268</x:v>
+      </x:c>
+      <x:c r="C48" t="s">
+        <x:v>269</x:v>
+      </x:c>
+      <x:c r="D48" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="E48" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="F48" t="n">
+        <x:f>SUM(F2:F47)</x:f>
+        <x:v>50.5</x:v>
+      </x:c>
+      <x:c r="G48"/>
+      <x:c r="H48"/>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="R8948ad81e54647bf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="R6eb60fc1d155419a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="R7afa2c26062d49d8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="R223061ab31424661"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="Rdbb6be92395240c4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="R15ad320e6cf3469f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="Rcd1c188cbde94bc6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R287cfc8c099a44ba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="Re7156d781c614d0b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="R18c4cbc952e54be2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R050ae36932384e3c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="R95295066d22c466f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="R4e3875c624144efb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="R21d3106a01114653"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R13b9282f5ba04538"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="Rb6182951caea4a98"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R7a7cd4209c6d4dd4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="R4aea3d8069ba40ad"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="R0164dc196a7f4a63"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="R03dee6570cb44257"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="Rd3d871f9fbd747ee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="R980700be606e4197"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="R02e6f8e175cc4759"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="Rc19c7d7cb628465a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="R7f22ef68c0114cb7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R27693db50f744947"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="R08150e4aba8a4d33"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="Rddaadef54ca24c2a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R71c9a4b6a6ff4dd6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="Rddaf22efb86b470c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="R927467403e534e1a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R98d14cc908534916"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="Re7bb6d4656b047f4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Rddceac87d9744eae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="Re77ef0309a6a44ca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R8b10a508ec0d437b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="Rb69d893bf56143c1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R6586ed1dade04db2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="Re56a5c2acf6a42ee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="Rd87ed6d380c34cba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="R21445e2f690c40d2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="R8e7d2872e021405a"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3231,688 +3430,688 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="9" t="s">
-        <x:v>243</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="B1" s="9" t="s">
-        <x:v>244</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="C1" s="9" t="s">
-        <x:v>245</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="D1" s="9" t="s">
-        <x:v>246</x:v>
+        <x:v>273</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="5" t="s">
-        <x:v>247</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="B2" s="5" t="s">
-        <x:v>248</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="C2" s="5" t="s">
-        <x:v>249</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="D2" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="s">
-        <x:v>251</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="B3" s="5" t="s">
-        <x:v>252</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="C3" s="5" t="s">
-        <x:v>253</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="D3" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>31</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C4" s="5" t="s">
-        <x:v>254</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="D4" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>255</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>256</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D6" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>44</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>257</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="D7" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>51</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>258</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="D8" s="6" t="s">
-        <x:v>250</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="66.25" customHeight="1">
+        <x:v>277</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="88.25" customHeight="1">
       <x:c r="A9" s="5" t="s">
-        <x:v>52</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B9" s="5" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C9" s="5" t="s">
-        <x:v>259</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="D9" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="5" t="s">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>260</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>261</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="D10" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="5" t="s">
-        <x:v>63</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B11" s="5" t="s">
-        <x:v>262</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="C11" s="5" t="s">
-        <x:v>263</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="D11" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>70</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>264</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="D12" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C13" s="5" t="s">
-        <x:v>265</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="D13" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D14" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
-        <x:v>79</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C15" s="5" t="s">
-        <x:v>80</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D15" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="5" t="s">
-        <x:v>82</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
-        <x:v>83</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
-        <x:v>84</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="D16" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="5" t="s">
-        <x:v>114</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B17" s="5" t="s">
-        <x:v>115</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C17" s="5" t="s">
-        <x:v>116</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="D17" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="5" t="s">
-        <x:v>86</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
-        <x:v>120</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="C18" s="5" t="s">
-        <x:v>266</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="D18" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="5" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
-        <x:v>92</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C19" s="5" t="s">
-        <x:v>267</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="D19" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="5" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
-        <x:v>124</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C20" s="5" t="s">
-        <x:v>268</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="D20" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="5" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B21" s="5" t="s">
-        <x:v>95</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C21" s="5" t="s">
-        <x:v>269</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="D21" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
-        <x:v>127</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C22" s="5" t="s">
-        <x:v>270</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="D22" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C23" s="5" t="s">
-        <x:v>271</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="D23" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
-        <x:v>133</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C24" s="5" t="s">
-        <x:v>272</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="D24" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
-        <x:v>99</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C25" s="5" t="s">
-        <x:v>273</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="D25" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B26" s="5" t="s">
-        <x:v>103</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C26" s="5" t="s">
-        <x:v>274</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="D26" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B27" s="5" t="s">
-        <x:v>136</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C27" s="5" t="s">
-        <x:v>275</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="D27" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B28" s="5" t="s">
-        <x:v>139</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C28" s="5" t="s">
-        <x:v>276</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="D28" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B29" s="5" t="s">
-        <x:v>142</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="C29" s="5" t="s">
-        <x:v>277</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="D29" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B30" s="5" t="s">
-        <x:v>145</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C30" s="5" t="s">
-        <x:v>278</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="D30" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B31" s="5" t="s">
-        <x:v>148</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C31" s="5" t="s">
-        <x:v>279</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="D31" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B32" s="5" t="s">
-        <x:v>150</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="C32" s="5" t="s">
-        <x:v>280</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="D32" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B33" s="5" t="s">
-        <x:v>153</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="C33" s="5" t="s">
-        <x:v>281</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="D33" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="5" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B34" s="5" t="s">
-        <x:v>107</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C34" s="5" t="s">
-        <x:v>282</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="D34" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="5" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B35" s="5" t="s">
-        <x:v>156</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="C35" s="5" t="s">
-        <x:v>283</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="D35" s="6" t="s">
-        <x:v>250</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="35.75" customHeight="1">
+        <x:v>277</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="47.75" customHeight="1">
       <x:c r="A36" s="5" t="s">
-        <x:v>159</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B36" s="5" t="s">
-        <x:v>160</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="C36" s="5" t="s">
-        <x:v>284</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="D36" s="14" t="s">
-        <x:v>250</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="35.75" customHeight="1">
+        <x:v>277</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="47.75" customHeight="1">
       <x:c r="A37" s="5" t="s">
-        <x:v>159</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B37" s="5" t="s">
-        <x:v>163</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="C37" s="5" t="s">
-        <x:v>285</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="D37" s="14" t="s">
-        <x:v>250</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="35.75" customHeight="1">
+        <x:v>277</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="47.75" customHeight="1">
       <x:c r="A38" s="5" t="s">
-        <x:v>168</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B38" s="5" t="s">
-        <x:v>169</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="C38" s="5" t="s">
-        <x:v>286</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="D38" s="14" t="s">
-        <x:v>250</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="35.75" customHeight="1">
+        <x:v>277</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="47.75" customHeight="1">
       <x:c r="A39" s="5" t="s">
-        <x:v>168</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B39" s="5" t="s">
-        <x:v>176</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C39" s="5" t="s">
-        <x:v>287</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="D39" s="14" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="s">
-        <x:v>235</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="B40" t="s">
-        <x:v>236</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="C40" t="s">
-        <x:v>288</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="D40" t="s">
-        <x:v>250</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="s">
-        <x:v>235</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="B41" t="s">
-        <x:v>240</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="C41" t="s">
-        <x:v>289</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="D41" t="s">
+        <x:v>277</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="B42" t="s">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="C42" t="s">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="D42" t="s">
+        <x:v>277</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="B43" t="s">
         <x:v>250</x:v>
       </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="B42" t="str">
-        <x:v>修正後の修正③</x:v>
-      </x:c>
-      <x:c r="C42" t="str">
-        <x:v>サーマニードルEVO同意書、ララドクター詳細・料金表・施術不可条件の修正</x:v>
-      </x:c>
-      <x:c r="D42" t="str">
-        <x:v>メールを開く</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="B43" t="str">
-        <x:v>修正後の修正④</x:v>
-      </x:c>
-      <x:c r="C43" t="str">
-        <x:v>美肌治療ページのスマホ表題を短縮・改行調整</x:v>
-      </x:c>
-      <x:c r="D43" t="str">
-        <x:v>メールを開く</x:v>
+      <x:c r="C43" t="s">
+        <x:v>318</x:v>
+      </x:c>
+      <x:c r="D43" t="s">
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="B44" t="str">
-        <x:v>修正後の修正⑤</x:v>
-      </x:c>
-      <x:c r="C44" t="str">
-        <x:v>説明・同意書表記、保護者同意書カード文言の統一</x:v>
-      </x:c>
-      <x:c r="D44" t="str">
-        <x:v>メールを開く</x:v>
+      <x:c r="A44" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="B44" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="C44" t="s">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="D44" t="s">
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="B45" t="str">
-        <x:v>修正後の修正⑥</x:v>
-      </x:c>
-      <x:c r="C45" t="str">
-        <x:v>マッサージピール・リバースピールのホームケア表示調整</x:v>
-      </x:c>
-      <x:c r="D45" t="str">
-        <x:v>メールを開く</x:v>
+      <x:c r="A45" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="B45" t="s">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C45" t="s">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="D45" t="s">
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" t="str">
-        <x:v>2026-07-27</x:v>
-      </x:c>
-      <x:c r="B46" t="str">
-        <x:v>修正後の修正⑦</x:v>
-      </x:c>
-      <x:c r="C46" t="str">
-        <x:v>問診票PDF、同意書リンク、ララドクターMENU／表題の修正</x:v>
-      </x:c>
-      <x:c r="D46" t="str">
-        <x:v>メールを開く</x:v>
+      <x:c r="A46" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="B46" t="s">
+        <x:v>260</x:v>
+      </x:c>
+      <x:c r="C46" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="D46" t="s">
+        <x:v>277</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="R5155592705e245c2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="Rf3af91e42fb34901"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R18470af760504b2d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="R0943f9a30dba4dec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="R585b4cad69354a1b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="R9d1b356a760543d1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="R2e01d50437e74d59"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="R40bd62aec41e4bc1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="Rb2144cf7edc347db"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="R3e7e17c5d3834af6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="R635d924e67d14b26"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="Rd1c0a2a6cc8a401e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="Rc56933de1f854686"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="Rdf6b6c4552c145d2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="R95d3ce120ddf4e9a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="Ra318fce15ff14c64"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="R48ce631bcd5e4504"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="Re0dad960425f44d5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="Rf52be63597ba47ef"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="Rced6b3f3c8df46b3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="R0a635703001d4479"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="R570a27ce75cc4bef"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="R9ab2adfbe3884d1b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="Re1bddbff65fb4551"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="Rcd737ca30f724bad"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="Ra3d3e5a81de04693"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="Re92f3538f9ae43bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="Rb81c42198e054b79"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="R148a96481bcb4773"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="Rfc86c49535a94960"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="R31b6008a7fb14859"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="Ra8b94f5aae9b4fc1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="Rdab6d07ea8184a45"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="Rd5b1ee9aff8e4205"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="R00e12b6069314e82"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="R1ed982d3613a4b1e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="Rbed878b894d84fbd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="R305526fe2e7141c5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="R840602dfb5b14266"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="R6b70375502254398"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="Re3c0d882c9e44ff6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="R2d48ec7939fb4fb2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="Rb087f0a326814a9a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="Rab317bc8eaf9406b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="Rc8110e94cd2f451f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="R9b810b7cb60a4d45"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="Rf387d0aa63dd4e29"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="Rf547064634584f21"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="R46d74f940d3a40ea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="R1bc5923232b0414e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="R26caf026892a4392"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="Rfb5eb6b72cb247ae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="R46b3c2ba640b4598"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="Rae5615c3349e4a60"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="R81e768b0efc947d8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="R6d281b2c57db49e4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="Rbfe085dc44574fe2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="Rc39a0b3c358f49e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="R51e59d65588a4988"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="R77847cef82f14447"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="R5f0efde1cb3a4754"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="R5c7f150b4b4b4e35"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="Rec06637a6fd143e4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="R35ed814c709a4f97"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="R6bb9c23dc20b4a5f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="Rba13476c2adf4c35"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="R95b86031ec2b4898"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="R1d4eec02513d48e3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="R06110a8fd24e401b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="R3cbb021750f2468b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="R41005e862283463b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="R87a8bb7411eb4090"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="R0cf46c65d3ec4bf9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="R1958ab8a601345a0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="R5d69c73545fb4d3d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="Rd5a2f83a25a24206"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>